<commit_message>
Remove emojis for a cleaner, professional look
</commit_message>
<xml_diff>
--- a/tracker/excel/LineShine_Tracker.xlsx
+++ b/tracker/excel/LineShine_Tracker.xlsx
@@ -596,13 +596,37 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="24">
     <dxf>
       <font>
         <name val="Arial"/>
         <b val="1"/>
         <color rgb="00027A48"/>
         <sz val="20"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00D92D20"/>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00B54708"/>
+        <sz val="16"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00027A48"/>
+        <sz val="16"/>
       </font>
     </dxf>
     <dxf>
@@ -2297,7 +2321,7 @@
         <v/>
       </c>
       <c r="D12" s="24">
-        <f>IF(A9+G9&gt;0,"🔴 At risk",IF(B13+0.15&lt;B12,"🟠 Behind schedule","🟢 On track"))</f>
+        <f>IF(A9+G9&gt;0,"AT RISK",IF(B13+0.15&lt;B12,"BEHIND SCHEDULE","ON TRACK"))</f>
         <v/>
       </c>
       <c r="J12" s="25" t="inlineStr">
@@ -3429,40 +3453,51 @@
       </dataBar>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D12">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>"AT RISK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
+      <formula>"BEHIND SCHEDULE"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
+      <formula>"ON TRACK"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="B19">
-    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="1">
+    <cfRule type="cellIs" priority="8" operator="greaterThan" dxfId="4">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G17:G24">
-    <cfRule type="expression" priority="6" dxfId="2">
+    <cfRule type="expression" priority="9" dxfId="5">
       <formula>AND(G17&lt;&gt;"",G17&lt;NOW())</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L17:L24">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="6">
       <formula>"Not started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="7">
       <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="8">
       <formula>"In review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="9">
       <formula>"Blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="10">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D48:D57">
-    <cfRule type="cellIs" priority="12" operator="greaterThan" dxfId="8">
+    <cfRule type="cellIs" priority="15" operator="greaterThan" dxfId="11">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G48:G57">
-    <cfRule type="dataBar" priority="13">
+    <cfRule type="dataBar" priority="16">
       <dataBar>
         <cfvo type="num" val="0"/>
         <cfvo type="num" val="1"/>
@@ -3471,7 +3506,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B48:B57">
-    <cfRule type="dataBar" priority="14">
+    <cfRule type="dataBar" priority="17">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -3624,7 +3659,7 @@
       </c>
       <c r="K7" s="51" t="inlineStr">
         <is>
-          <t>😀 Great</t>
+          <t>Great</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3697,7 @@
       </c>
       <c r="K8" s="51" t="inlineStr">
         <is>
-          <t>🙂 Good</t>
+          <t>Good</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3735,7 @@
       </c>
       <c r="K9" s="51" t="inlineStr">
         <is>
-          <t>😐 OK</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -3732,7 +3767,7 @@
       <c r="J10" s="51" t="n"/>
       <c r="K10" s="51" t="inlineStr">
         <is>
-          <t>🙁 Struggling</t>
+          <t>Struggling</t>
         </is>
       </c>
     </row>
@@ -3866,7 +3901,7 @@
       <c r="D18" s="56" t="n"/>
       <c r="F18" s="57" t="inlineStr">
         <is>
-          <t>⚠ Task status 'Done' and 'Blocked' are used by formulas: rename them only together with the formulas.</t>
+          <t>Note: task status 'Done' and 'Blocked' are used by formulas: rename them only together with the formulas.</t>
         </is>
       </c>
     </row>
@@ -4120,7 +4155,7 @@
         <v/>
       </c>
       <c r="M6" s="58">
-        <f>IF(B6="","",IF(E6="Done","✓ Done",IF(E6="Blocked","Blocked",IF(H6="","No due date",IF(H6&lt;NOW(),"Overdue",IF(H6-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B6="","",IF(E6="Done","Complete",IF(E6="Blocked","Blocked",IF(H6="","No due date",IF(H6&lt;NOW(),"Overdue",IF(H6-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N6" s="51" t="n"/>
@@ -4174,7 +4209,7 @@
         <v/>
       </c>
       <c r="M7" s="58">
-        <f>IF(B7="","",IF(E7="Done","✓ Done",IF(E7="Blocked","Blocked",IF(H7="","No due date",IF(H7&lt;NOW(),"Overdue",IF(H7-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B7="","",IF(E7="Done","Complete",IF(E7="Blocked","Blocked",IF(H7="","No due date",IF(H7&lt;NOW(),"Overdue",IF(H7-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N7" s="51" t="n"/>
@@ -4232,7 +4267,7 @@
         <v/>
       </c>
       <c r="M8" s="58">
-        <f>IF(B8="","",IF(E8="Done","✓ Done",IF(E8="Blocked","Blocked",IF(H8="","No due date",IF(H8&lt;NOW(),"Overdue",IF(H8-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B8="","",IF(E8="Done","Complete",IF(E8="Blocked","Blocked",IF(H8="","No due date",IF(H8&lt;NOW(),"Overdue",IF(H8-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N8" s="51" t="n"/>
@@ -4290,7 +4325,7 @@
         <v/>
       </c>
       <c r="M9" s="58">
-        <f>IF(B9="","",IF(E9="Done","✓ Done",IF(E9="Blocked","Blocked",IF(H9="","No due date",IF(H9&lt;NOW(),"Overdue",IF(H9-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B9="","",IF(E9="Done","Complete",IF(E9="Blocked","Blocked",IF(H9="","No due date",IF(H9&lt;NOW(),"Overdue",IF(H9-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N9" s="51" t="n"/>
@@ -4348,7 +4383,7 @@
         <v/>
       </c>
       <c r="M10" s="58">
-        <f>IF(B10="","",IF(E10="Done","✓ Done",IF(E10="Blocked","Blocked",IF(H10="","No due date",IF(H10&lt;NOW(),"Overdue",IF(H10-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B10="","",IF(E10="Done","Complete",IF(E10="Blocked","Blocked",IF(H10="","No due date",IF(H10&lt;NOW(),"Overdue",IF(H10-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N10" s="51" t="n"/>
@@ -4406,7 +4441,7 @@
         <v/>
       </c>
       <c r="M11" s="58">
-        <f>IF(B11="","",IF(E11="Done","✓ Done",IF(E11="Blocked","Blocked",IF(H11="","No due date",IF(H11&lt;NOW(),"Overdue",IF(H11-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B11="","",IF(E11="Done","Complete",IF(E11="Blocked","Blocked",IF(H11="","No due date",IF(H11&lt;NOW(),"Overdue",IF(H11-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N11" s="51" t="n"/>
@@ -4464,7 +4499,7 @@
         <v/>
       </c>
       <c r="M12" s="58">
-        <f>IF(B12="","",IF(E12="Done","✓ Done",IF(E12="Blocked","Blocked",IF(H12="","No due date",IF(H12&lt;NOW(),"Overdue",IF(H12-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B12="","",IF(E12="Done","Complete",IF(E12="Blocked","Blocked",IF(H12="","No due date",IF(H12&lt;NOW(),"Overdue",IF(H12-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N12" s="51" t="n"/>
@@ -4522,7 +4557,7 @@
         <v/>
       </c>
       <c r="M13" s="58">
-        <f>IF(B13="","",IF(E13="Done","✓ Done",IF(E13="Blocked","Blocked",IF(H13="","No due date",IF(H13&lt;NOW(),"Overdue",IF(H13-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B13="","",IF(E13="Done","Complete",IF(E13="Blocked","Blocked",IF(H13="","No due date",IF(H13&lt;NOW(),"Overdue",IF(H13-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N13" s="51" t="n"/>
@@ -4580,7 +4615,7 @@
         <v/>
       </c>
       <c r="M14" s="58">
-        <f>IF(B14="","",IF(E14="Done","✓ Done",IF(E14="Blocked","Blocked",IF(H14="","No due date",IF(H14&lt;NOW(),"Overdue",IF(H14-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B14="","",IF(E14="Done","Complete",IF(E14="Blocked","Blocked",IF(H14="","No due date",IF(H14&lt;NOW(),"Overdue",IF(H14-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N14" s="51" t="n"/>
@@ -4636,7 +4671,7 @@
         <v/>
       </c>
       <c r="M15" s="58">
-        <f>IF(B15="","",IF(E15="Done","✓ Done",IF(E15="Blocked","Blocked",IF(H15="","No due date",IF(H15&lt;NOW(),"Overdue",IF(H15-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B15="","",IF(E15="Done","Complete",IF(E15="Blocked","Blocked",IF(H15="","No due date",IF(H15&lt;NOW(),"Overdue",IF(H15-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N15" s="51" t="n"/>
@@ -4688,7 +4723,7 @@
         <v/>
       </c>
       <c r="M16" s="58">
-        <f>IF(B16="","",IF(E16="Done","✓ Done",IF(E16="Blocked","Blocked",IF(H16="","No due date",IF(H16&lt;NOW(),"Overdue",IF(H16-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B16="","",IF(E16="Done","Complete",IF(E16="Blocked","Blocked",IF(H16="","No due date",IF(H16&lt;NOW(),"Overdue",IF(H16-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N16" s="51" t="n"/>
@@ -4742,7 +4777,7 @@
         <v/>
       </c>
       <c r="M17" s="58">
-        <f>IF(B17="","",IF(E17="Done","✓ Done",IF(E17="Blocked","Blocked",IF(H17="","No due date",IF(H17&lt;NOW(),"Overdue",IF(H17-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B17="","",IF(E17="Done","Complete",IF(E17="Blocked","Blocked",IF(H17="","No due date",IF(H17&lt;NOW(),"Overdue",IF(H17-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N17" s="51" t="n"/>
@@ -4772,7 +4807,7 @@
         <v/>
       </c>
       <c r="M18" s="58">
-        <f>IF(B18="","",IF(E18="Done","✓ Done",IF(E18="Blocked","Blocked",IF(H18="","No due date",IF(H18&lt;NOW(),"Overdue",IF(H18-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B18="","",IF(E18="Done","Complete",IF(E18="Blocked","Blocked",IF(H18="","No due date",IF(H18&lt;NOW(),"Overdue",IF(H18-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N18" s="51" t="n"/>
@@ -4802,7 +4837,7 @@
         <v/>
       </c>
       <c r="M19" s="58">
-        <f>IF(B19="","",IF(E19="Done","✓ Done",IF(E19="Blocked","Blocked",IF(H19="","No due date",IF(H19&lt;NOW(),"Overdue",IF(H19-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B19="","",IF(E19="Done","Complete",IF(E19="Blocked","Blocked",IF(H19="","No due date",IF(H19&lt;NOW(),"Overdue",IF(H19-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N19" s="51" t="n"/>
@@ -4832,7 +4867,7 @@
         <v/>
       </c>
       <c r="M20" s="58">
-        <f>IF(B20="","",IF(E20="Done","✓ Done",IF(E20="Blocked","Blocked",IF(H20="","No due date",IF(H20&lt;NOW(),"Overdue",IF(H20-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B20="","",IF(E20="Done","Complete",IF(E20="Blocked","Blocked",IF(H20="","No due date",IF(H20&lt;NOW(),"Overdue",IF(H20-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N20" s="51" t="n"/>
@@ -4862,7 +4897,7 @@
         <v/>
       </c>
       <c r="M21" s="58">
-        <f>IF(B21="","",IF(E21="Done","✓ Done",IF(E21="Blocked","Blocked",IF(H21="","No due date",IF(H21&lt;NOW(),"Overdue",IF(H21-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B21="","",IF(E21="Done","Complete",IF(E21="Blocked","Blocked",IF(H21="","No due date",IF(H21&lt;NOW(),"Overdue",IF(H21-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N21" s="51" t="n"/>
@@ -4892,7 +4927,7 @@
         <v/>
       </c>
       <c r="M22" s="58">
-        <f>IF(B22="","",IF(E22="Done","✓ Done",IF(E22="Blocked","Blocked",IF(H22="","No due date",IF(H22&lt;NOW(),"Overdue",IF(H22-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B22="","",IF(E22="Done","Complete",IF(E22="Blocked","Blocked",IF(H22="","No due date",IF(H22&lt;NOW(),"Overdue",IF(H22-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N22" s="51" t="n"/>
@@ -4922,7 +4957,7 @@
         <v/>
       </c>
       <c r="M23" s="58">
-        <f>IF(B23="","",IF(E23="Done","✓ Done",IF(E23="Blocked","Blocked",IF(H23="","No due date",IF(H23&lt;NOW(),"Overdue",IF(H23-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B23="","",IF(E23="Done","Complete",IF(E23="Blocked","Blocked",IF(H23="","No due date",IF(H23&lt;NOW(),"Overdue",IF(H23-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N23" s="51" t="n"/>
@@ -4952,7 +4987,7 @@
         <v/>
       </c>
       <c r="M24" s="58">
-        <f>IF(B24="","",IF(E24="Done","✓ Done",IF(E24="Blocked","Blocked",IF(H24="","No due date",IF(H24&lt;NOW(),"Overdue",IF(H24-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B24="","",IF(E24="Done","Complete",IF(E24="Blocked","Blocked",IF(H24="","No due date",IF(H24&lt;NOW(),"Overdue",IF(H24-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N24" s="51" t="n"/>
@@ -4982,7 +5017,7 @@
         <v/>
       </c>
       <c r="M25" s="58">
-        <f>IF(B25="","",IF(E25="Done","✓ Done",IF(E25="Blocked","Blocked",IF(H25="","No due date",IF(H25&lt;NOW(),"Overdue",IF(H25-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B25="","",IF(E25="Done","Complete",IF(E25="Blocked","Blocked",IF(H25="","No due date",IF(H25&lt;NOW(),"Overdue",IF(H25-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N25" s="51" t="n"/>
@@ -5012,7 +5047,7 @@
         <v/>
       </c>
       <c r="M26" s="58">
-        <f>IF(B26="","",IF(E26="Done","✓ Done",IF(E26="Blocked","Blocked",IF(H26="","No due date",IF(H26&lt;NOW(),"Overdue",IF(H26-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B26="","",IF(E26="Done","Complete",IF(E26="Blocked","Blocked",IF(H26="","No due date",IF(H26&lt;NOW(),"Overdue",IF(H26-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N26" s="51" t="n"/>
@@ -5042,7 +5077,7 @@
         <v/>
       </c>
       <c r="M27" s="58">
-        <f>IF(B27="","",IF(E27="Done","✓ Done",IF(E27="Blocked","Blocked",IF(H27="","No due date",IF(H27&lt;NOW(),"Overdue",IF(H27-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B27="","",IF(E27="Done","Complete",IF(E27="Blocked","Blocked",IF(H27="","No due date",IF(H27&lt;NOW(),"Overdue",IF(H27-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N27" s="51" t="n"/>
@@ -5072,7 +5107,7 @@
         <v/>
       </c>
       <c r="M28" s="58">
-        <f>IF(B28="","",IF(E28="Done","✓ Done",IF(E28="Blocked","Blocked",IF(H28="","No due date",IF(H28&lt;NOW(),"Overdue",IF(H28-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B28="","",IF(E28="Done","Complete",IF(E28="Blocked","Blocked",IF(H28="","No due date",IF(H28&lt;NOW(),"Overdue",IF(H28-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N28" s="51" t="n"/>
@@ -5102,7 +5137,7 @@
         <v/>
       </c>
       <c r="M29" s="58">
-        <f>IF(B29="","",IF(E29="Done","✓ Done",IF(E29="Blocked","Blocked",IF(H29="","No due date",IF(H29&lt;NOW(),"Overdue",IF(H29-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B29="","",IF(E29="Done","Complete",IF(E29="Blocked","Blocked",IF(H29="","No due date",IF(H29&lt;NOW(),"Overdue",IF(H29-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N29" s="51" t="n"/>
@@ -5132,7 +5167,7 @@
         <v/>
       </c>
       <c r="M30" s="58">
-        <f>IF(B30="","",IF(E30="Done","✓ Done",IF(E30="Blocked","Blocked",IF(H30="","No due date",IF(H30&lt;NOW(),"Overdue",IF(H30-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B30="","",IF(E30="Done","Complete",IF(E30="Blocked","Blocked",IF(H30="","No due date",IF(H30&lt;NOW(),"Overdue",IF(H30-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N30" s="51" t="n"/>
@@ -5162,7 +5197,7 @@
         <v/>
       </c>
       <c r="M31" s="58">
-        <f>IF(B31="","",IF(E31="Done","✓ Done",IF(E31="Blocked","Blocked",IF(H31="","No due date",IF(H31&lt;NOW(),"Overdue",IF(H31-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B31="","",IF(E31="Done","Complete",IF(E31="Blocked","Blocked",IF(H31="","No due date",IF(H31&lt;NOW(),"Overdue",IF(H31-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N31" s="51" t="n"/>
@@ -5192,7 +5227,7 @@
         <v/>
       </c>
       <c r="M32" s="58">
-        <f>IF(B32="","",IF(E32="Done","✓ Done",IF(E32="Blocked","Blocked",IF(H32="","No due date",IF(H32&lt;NOW(),"Overdue",IF(H32-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B32="","",IF(E32="Done","Complete",IF(E32="Blocked","Blocked",IF(H32="","No due date",IF(H32&lt;NOW(),"Overdue",IF(H32-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N32" s="51" t="n"/>
@@ -5222,7 +5257,7 @@
         <v/>
       </c>
       <c r="M33" s="58">
-        <f>IF(B33="","",IF(E33="Done","✓ Done",IF(E33="Blocked","Blocked",IF(H33="","No due date",IF(H33&lt;NOW(),"Overdue",IF(H33-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B33="","",IF(E33="Done","Complete",IF(E33="Blocked","Blocked",IF(H33="","No due date",IF(H33&lt;NOW(),"Overdue",IF(H33-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N33" s="51" t="n"/>
@@ -5252,7 +5287,7 @@
         <v/>
       </c>
       <c r="M34" s="58">
-        <f>IF(B34="","",IF(E34="Done","✓ Done",IF(E34="Blocked","Blocked",IF(H34="","No due date",IF(H34&lt;NOW(),"Overdue",IF(H34-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B34="","",IF(E34="Done","Complete",IF(E34="Blocked","Blocked",IF(H34="","No due date",IF(H34&lt;NOW(),"Overdue",IF(H34-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N34" s="51" t="n"/>
@@ -5282,7 +5317,7 @@
         <v/>
       </c>
       <c r="M35" s="58">
-        <f>IF(B35="","",IF(E35="Done","✓ Done",IF(E35="Blocked","Blocked",IF(H35="","No due date",IF(H35&lt;NOW(),"Overdue",IF(H35-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B35="","",IF(E35="Done","Complete",IF(E35="Blocked","Blocked",IF(H35="","No due date",IF(H35&lt;NOW(),"Overdue",IF(H35-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N35" s="51" t="n"/>
@@ -5312,7 +5347,7 @@
         <v/>
       </c>
       <c r="M36" s="58">
-        <f>IF(B36="","",IF(E36="Done","✓ Done",IF(E36="Blocked","Blocked",IF(H36="","No due date",IF(H36&lt;NOW(),"Overdue",IF(H36-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B36="","",IF(E36="Done","Complete",IF(E36="Blocked","Blocked",IF(H36="","No due date",IF(H36&lt;NOW(),"Overdue",IF(H36-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N36" s="51" t="n"/>
@@ -5342,7 +5377,7 @@
         <v/>
       </c>
       <c r="M37" s="58">
-        <f>IF(B37="","",IF(E37="Done","✓ Done",IF(E37="Blocked","Blocked",IF(H37="","No due date",IF(H37&lt;NOW(),"Overdue",IF(H37-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B37="","",IF(E37="Done","Complete",IF(E37="Blocked","Blocked",IF(H37="","No due date",IF(H37&lt;NOW(),"Overdue",IF(H37-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N37" s="51" t="n"/>
@@ -5372,7 +5407,7 @@
         <v/>
       </c>
       <c r="M38" s="58">
-        <f>IF(B38="","",IF(E38="Done","✓ Done",IF(E38="Blocked","Blocked",IF(H38="","No due date",IF(H38&lt;NOW(),"Overdue",IF(H38-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B38="","",IF(E38="Done","Complete",IF(E38="Blocked","Blocked",IF(H38="","No due date",IF(H38&lt;NOW(),"Overdue",IF(H38-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N38" s="51" t="n"/>
@@ -5402,7 +5437,7 @@
         <v/>
       </c>
       <c r="M39" s="58">
-        <f>IF(B39="","",IF(E39="Done","✓ Done",IF(E39="Blocked","Blocked",IF(H39="","No due date",IF(H39&lt;NOW(),"Overdue",IF(H39-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B39="","",IF(E39="Done","Complete",IF(E39="Blocked","Blocked",IF(H39="","No due date",IF(H39&lt;NOW(),"Overdue",IF(H39-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N39" s="51" t="n"/>
@@ -5432,7 +5467,7 @@
         <v/>
       </c>
       <c r="M40" s="58">
-        <f>IF(B40="","",IF(E40="Done","✓ Done",IF(E40="Blocked","Blocked",IF(H40="","No due date",IF(H40&lt;NOW(),"Overdue",IF(H40-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B40="","",IF(E40="Done","Complete",IF(E40="Blocked","Blocked",IF(H40="","No due date",IF(H40&lt;NOW(),"Overdue",IF(H40-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N40" s="51" t="n"/>
@@ -5462,7 +5497,7 @@
         <v/>
       </c>
       <c r="M41" s="58">
-        <f>IF(B41="","",IF(E41="Done","✓ Done",IF(E41="Blocked","Blocked",IF(H41="","No due date",IF(H41&lt;NOW(),"Overdue",IF(H41-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B41="","",IF(E41="Done","Complete",IF(E41="Blocked","Blocked",IF(H41="","No due date",IF(H41&lt;NOW(),"Overdue",IF(H41-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N41" s="51" t="n"/>
@@ -5492,7 +5527,7 @@
         <v/>
       </c>
       <c r="M42" s="58">
-        <f>IF(B42="","",IF(E42="Done","✓ Done",IF(E42="Blocked","Blocked",IF(H42="","No due date",IF(H42&lt;NOW(),"Overdue",IF(H42-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B42="","",IF(E42="Done","Complete",IF(E42="Blocked","Blocked",IF(H42="","No due date",IF(H42&lt;NOW(),"Overdue",IF(H42-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N42" s="51" t="n"/>
@@ -5522,7 +5557,7 @@
         <v/>
       </c>
       <c r="M43" s="58">
-        <f>IF(B43="","",IF(E43="Done","✓ Done",IF(E43="Blocked","Blocked",IF(H43="","No due date",IF(H43&lt;NOW(),"Overdue",IF(H43-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B43="","",IF(E43="Done","Complete",IF(E43="Blocked","Blocked",IF(H43="","No due date",IF(H43&lt;NOW(),"Overdue",IF(H43-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N43" s="51" t="n"/>
@@ -5552,7 +5587,7 @@
         <v/>
       </c>
       <c r="M44" s="58">
-        <f>IF(B44="","",IF(E44="Done","✓ Done",IF(E44="Blocked","Blocked",IF(H44="","No due date",IF(H44&lt;NOW(),"Overdue",IF(H44-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B44="","",IF(E44="Done","Complete",IF(E44="Blocked","Blocked",IF(H44="","No due date",IF(H44&lt;NOW(),"Overdue",IF(H44-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N44" s="51" t="n"/>
@@ -5582,7 +5617,7 @@
         <v/>
       </c>
       <c r="M45" s="58">
-        <f>IF(B45="","",IF(E45="Done","✓ Done",IF(E45="Blocked","Blocked",IF(H45="","No due date",IF(H45&lt;NOW(),"Overdue",IF(H45-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B45="","",IF(E45="Done","Complete",IF(E45="Blocked","Blocked",IF(H45="","No due date",IF(H45&lt;NOW(),"Overdue",IF(H45-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N45" s="51" t="n"/>
@@ -5612,7 +5647,7 @@
         <v/>
       </c>
       <c r="M46" s="58">
-        <f>IF(B46="","",IF(E46="Done","✓ Done",IF(E46="Blocked","Blocked",IF(H46="","No due date",IF(H46&lt;NOW(),"Overdue",IF(H46-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B46="","",IF(E46="Done","Complete",IF(E46="Blocked","Blocked",IF(H46="","No due date",IF(H46&lt;NOW(),"Overdue",IF(H46-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N46" s="51" t="n"/>
@@ -5642,7 +5677,7 @@
         <v/>
       </c>
       <c r="M47" s="58">
-        <f>IF(B47="","",IF(E47="Done","✓ Done",IF(E47="Blocked","Blocked",IF(H47="","No due date",IF(H47&lt;NOW(),"Overdue",IF(H47-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B47="","",IF(E47="Done","Complete",IF(E47="Blocked","Blocked",IF(H47="","No due date",IF(H47&lt;NOW(),"Overdue",IF(H47-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N47" s="51" t="n"/>
@@ -5672,7 +5707,7 @@
         <v/>
       </c>
       <c r="M48" s="58">
-        <f>IF(B48="","",IF(E48="Done","✓ Done",IF(E48="Blocked","Blocked",IF(H48="","No due date",IF(H48&lt;NOW(),"Overdue",IF(H48-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B48="","",IF(E48="Done","Complete",IF(E48="Blocked","Blocked",IF(H48="","No due date",IF(H48&lt;NOW(),"Overdue",IF(H48-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N48" s="51" t="n"/>
@@ -5702,7 +5737,7 @@
         <v/>
       </c>
       <c r="M49" s="58">
-        <f>IF(B49="","",IF(E49="Done","✓ Done",IF(E49="Blocked","Blocked",IF(H49="","No due date",IF(H49&lt;NOW(),"Overdue",IF(H49-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B49="","",IF(E49="Done","Complete",IF(E49="Blocked","Blocked",IF(H49="","No due date",IF(H49&lt;NOW(),"Overdue",IF(H49-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N49" s="51" t="n"/>
@@ -5732,7 +5767,7 @@
         <v/>
       </c>
       <c r="M50" s="58">
-        <f>IF(B50="","",IF(E50="Done","✓ Done",IF(E50="Blocked","Blocked",IF(H50="","No due date",IF(H50&lt;NOW(),"Overdue",IF(H50-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B50="","",IF(E50="Done","Complete",IF(E50="Blocked","Blocked",IF(H50="","No due date",IF(H50&lt;NOW(),"Overdue",IF(H50-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N50" s="51" t="n"/>
@@ -5762,7 +5797,7 @@
         <v/>
       </c>
       <c r="M51" s="58">
-        <f>IF(B51="","",IF(E51="Done","✓ Done",IF(E51="Blocked","Blocked",IF(H51="","No due date",IF(H51&lt;NOW(),"Overdue",IF(H51-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B51="","",IF(E51="Done","Complete",IF(E51="Blocked","Blocked",IF(H51="","No due date",IF(H51&lt;NOW(),"Overdue",IF(H51-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N51" s="51" t="n"/>
@@ -5792,7 +5827,7 @@
         <v/>
       </c>
       <c r="M52" s="58">
-        <f>IF(B52="","",IF(E52="Done","✓ Done",IF(E52="Blocked","Blocked",IF(H52="","No due date",IF(H52&lt;NOW(),"Overdue",IF(H52-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B52="","",IF(E52="Done","Complete",IF(E52="Blocked","Blocked",IF(H52="","No due date",IF(H52&lt;NOW(),"Overdue",IF(H52-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N52" s="51" t="n"/>
@@ -5822,7 +5857,7 @@
         <v/>
       </c>
       <c r="M53" s="58">
-        <f>IF(B53="","",IF(E53="Done","✓ Done",IF(E53="Blocked","Blocked",IF(H53="","No due date",IF(H53&lt;NOW(),"Overdue",IF(H53-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B53="","",IF(E53="Done","Complete",IF(E53="Blocked","Blocked",IF(H53="","No due date",IF(H53&lt;NOW(),"Overdue",IF(H53-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N53" s="51" t="n"/>
@@ -5852,7 +5887,7 @@
         <v/>
       </c>
       <c r="M54" s="58">
-        <f>IF(B54="","",IF(E54="Done","✓ Done",IF(E54="Blocked","Blocked",IF(H54="","No due date",IF(H54&lt;NOW(),"Overdue",IF(H54-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B54="","",IF(E54="Done","Complete",IF(E54="Blocked","Blocked",IF(H54="","No due date",IF(H54&lt;NOW(),"Overdue",IF(H54-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N54" s="51" t="n"/>
@@ -5882,7 +5917,7 @@
         <v/>
       </c>
       <c r="M55" s="58">
-        <f>IF(B55="","",IF(E55="Done","✓ Done",IF(E55="Blocked","Blocked",IF(H55="","No due date",IF(H55&lt;NOW(),"Overdue",IF(H55-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B55="","",IF(E55="Done","Complete",IF(E55="Blocked","Blocked",IF(H55="","No due date",IF(H55&lt;NOW(),"Overdue",IF(H55-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N55" s="51" t="n"/>
@@ -5912,7 +5947,7 @@
         <v/>
       </c>
       <c r="M56" s="58">
-        <f>IF(B56="","",IF(E56="Done","✓ Done",IF(E56="Blocked","Blocked",IF(H56="","No due date",IF(H56&lt;NOW(),"Overdue",IF(H56-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B56="","",IF(E56="Done","Complete",IF(E56="Blocked","Blocked",IF(H56="","No due date",IF(H56&lt;NOW(),"Overdue",IF(H56-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N56" s="51" t="n"/>
@@ -5942,7 +5977,7 @@
         <v/>
       </c>
       <c r="M57" s="58">
-        <f>IF(B57="","",IF(E57="Done","✓ Done",IF(E57="Blocked","Blocked",IF(H57="","No due date",IF(H57&lt;NOW(),"Overdue",IF(H57-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B57="","",IF(E57="Done","Complete",IF(E57="Blocked","Blocked",IF(H57="","No due date",IF(H57&lt;NOW(),"Overdue",IF(H57-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N57" s="51" t="n"/>
@@ -5972,7 +6007,7 @@
         <v/>
       </c>
       <c r="M58" s="58">
-        <f>IF(B58="","",IF(E58="Done","✓ Done",IF(E58="Blocked","Blocked",IF(H58="","No due date",IF(H58&lt;NOW(),"Overdue",IF(H58-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B58="","",IF(E58="Done","Complete",IF(E58="Blocked","Blocked",IF(H58="","No due date",IF(H58&lt;NOW(),"Overdue",IF(H58-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N58" s="51" t="n"/>
@@ -6002,7 +6037,7 @@
         <v/>
       </c>
       <c r="M59" s="58">
-        <f>IF(B59="","",IF(E59="Done","✓ Done",IF(E59="Blocked","Blocked",IF(H59="","No due date",IF(H59&lt;NOW(),"Overdue",IF(H59-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B59="","",IF(E59="Done","Complete",IF(E59="Blocked","Blocked",IF(H59="","No due date",IF(H59&lt;NOW(),"Overdue",IF(H59-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N59" s="51" t="n"/>
@@ -6032,7 +6067,7 @@
         <v/>
       </c>
       <c r="M60" s="58">
-        <f>IF(B60="","",IF(E60="Done","✓ Done",IF(E60="Blocked","Blocked",IF(H60="","No due date",IF(H60&lt;NOW(),"Overdue",IF(H60-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B60="","",IF(E60="Done","Complete",IF(E60="Blocked","Blocked",IF(H60="","No due date",IF(H60&lt;NOW(),"Overdue",IF(H60-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N60" s="51" t="n"/>
@@ -6062,7 +6097,7 @@
         <v/>
       </c>
       <c r="M61" s="58">
-        <f>IF(B61="","",IF(E61="Done","✓ Done",IF(E61="Blocked","Blocked",IF(H61="","No due date",IF(H61&lt;NOW(),"Overdue",IF(H61-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B61="","",IF(E61="Done","Complete",IF(E61="Blocked","Blocked",IF(H61="","No due date",IF(H61&lt;NOW(),"Overdue",IF(H61-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N61" s="51" t="n"/>
@@ -6092,7 +6127,7 @@
         <v/>
       </c>
       <c r="M62" s="58">
-        <f>IF(B62="","",IF(E62="Done","✓ Done",IF(E62="Blocked","Blocked",IF(H62="","No due date",IF(H62&lt;NOW(),"Overdue",IF(H62-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B62="","",IF(E62="Done","Complete",IF(E62="Blocked","Blocked",IF(H62="","No due date",IF(H62&lt;NOW(),"Overdue",IF(H62-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N62" s="51" t="n"/>
@@ -6122,7 +6157,7 @@
         <v/>
       </c>
       <c r="M63" s="58">
-        <f>IF(B63="","",IF(E63="Done","✓ Done",IF(E63="Blocked","Blocked",IF(H63="","No due date",IF(H63&lt;NOW(),"Overdue",IF(H63-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B63="","",IF(E63="Done","Complete",IF(E63="Blocked","Blocked",IF(H63="","No due date",IF(H63&lt;NOW(),"Overdue",IF(H63-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N63" s="51" t="n"/>
@@ -6152,7 +6187,7 @@
         <v/>
       </c>
       <c r="M64" s="58">
-        <f>IF(B64="","",IF(E64="Done","✓ Done",IF(E64="Blocked","Blocked",IF(H64="","No due date",IF(H64&lt;NOW(),"Overdue",IF(H64-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B64="","",IF(E64="Done","Complete",IF(E64="Blocked","Blocked",IF(H64="","No due date",IF(H64&lt;NOW(),"Overdue",IF(H64-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N64" s="51" t="n"/>
@@ -6182,7 +6217,7 @@
         <v/>
       </c>
       <c r="M65" s="58">
-        <f>IF(B65="","",IF(E65="Done","✓ Done",IF(E65="Blocked","Blocked",IF(H65="","No due date",IF(H65&lt;NOW(),"Overdue",IF(H65-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B65="","",IF(E65="Done","Complete",IF(E65="Blocked","Blocked",IF(H65="","No due date",IF(H65&lt;NOW(),"Overdue",IF(H65-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N65" s="51" t="n"/>
@@ -6212,7 +6247,7 @@
         <v/>
       </c>
       <c r="M66" s="58">
-        <f>IF(B66="","",IF(E66="Done","✓ Done",IF(E66="Blocked","Blocked",IF(H66="","No due date",IF(H66&lt;NOW(),"Overdue",IF(H66-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B66="","",IF(E66="Done","Complete",IF(E66="Blocked","Blocked",IF(H66="","No due date",IF(H66&lt;NOW(),"Overdue",IF(H66-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N66" s="51" t="n"/>
@@ -6242,7 +6277,7 @@
         <v/>
       </c>
       <c r="M67" s="58">
-        <f>IF(B67="","",IF(E67="Done","✓ Done",IF(E67="Blocked","Blocked",IF(H67="","No due date",IF(H67&lt;NOW(),"Overdue",IF(H67-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B67="","",IF(E67="Done","Complete",IF(E67="Blocked","Blocked",IF(H67="","No due date",IF(H67&lt;NOW(),"Overdue",IF(H67-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N67" s="51" t="n"/>
@@ -6272,7 +6307,7 @@
         <v/>
       </c>
       <c r="M68" s="58">
-        <f>IF(B68="","",IF(E68="Done","✓ Done",IF(E68="Blocked","Blocked",IF(H68="","No due date",IF(H68&lt;NOW(),"Overdue",IF(H68-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B68="","",IF(E68="Done","Complete",IF(E68="Blocked","Blocked",IF(H68="","No due date",IF(H68&lt;NOW(),"Overdue",IF(H68-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N68" s="51" t="n"/>
@@ -6302,7 +6337,7 @@
         <v/>
       </c>
       <c r="M69" s="58">
-        <f>IF(B69="","",IF(E69="Done","✓ Done",IF(E69="Blocked","Blocked",IF(H69="","No due date",IF(H69&lt;NOW(),"Overdue",IF(H69-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B69="","",IF(E69="Done","Complete",IF(E69="Blocked","Blocked",IF(H69="","No due date",IF(H69&lt;NOW(),"Overdue",IF(H69-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N69" s="51" t="n"/>
@@ -6332,7 +6367,7 @@
         <v/>
       </c>
       <c r="M70" s="58">
-        <f>IF(B70="","",IF(E70="Done","✓ Done",IF(E70="Blocked","Blocked",IF(H70="","No due date",IF(H70&lt;NOW(),"Overdue",IF(H70-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B70="","",IF(E70="Done","Complete",IF(E70="Blocked","Blocked",IF(H70="","No due date",IF(H70&lt;NOW(),"Overdue",IF(H70-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N70" s="51" t="n"/>
@@ -6362,7 +6397,7 @@
         <v/>
       </c>
       <c r="M71" s="58">
-        <f>IF(B71="","",IF(E71="Done","✓ Done",IF(E71="Blocked","Blocked",IF(H71="","No due date",IF(H71&lt;NOW(),"Overdue",IF(H71-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B71="","",IF(E71="Done","Complete",IF(E71="Blocked","Blocked",IF(H71="","No due date",IF(H71&lt;NOW(),"Overdue",IF(H71-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N71" s="51" t="n"/>
@@ -6392,7 +6427,7 @@
         <v/>
       </c>
       <c r="M72" s="58">
-        <f>IF(B72="","",IF(E72="Done","✓ Done",IF(E72="Blocked","Blocked",IF(H72="","No due date",IF(H72&lt;NOW(),"Overdue",IF(H72-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B72="","",IF(E72="Done","Complete",IF(E72="Blocked","Blocked",IF(H72="","No due date",IF(H72&lt;NOW(),"Overdue",IF(H72-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N72" s="51" t="n"/>
@@ -6422,7 +6457,7 @@
         <v/>
       </c>
       <c r="M73" s="58">
-        <f>IF(B73="","",IF(E73="Done","✓ Done",IF(E73="Blocked","Blocked",IF(H73="","No due date",IF(H73&lt;NOW(),"Overdue",IF(H73-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B73="","",IF(E73="Done","Complete",IF(E73="Blocked","Blocked",IF(H73="","No due date",IF(H73&lt;NOW(),"Overdue",IF(H73-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N73" s="51" t="n"/>
@@ -6452,7 +6487,7 @@
         <v/>
       </c>
       <c r="M74" s="58">
-        <f>IF(B74="","",IF(E74="Done","✓ Done",IF(E74="Blocked","Blocked",IF(H74="","No due date",IF(H74&lt;NOW(),"Overdue",IF(H74-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B74="","",IF(E74="Done","Complete",IF(E74="Blocked","Blocked",IF(H74="","No due date",IF(H74&lt;NOW(),"Overdue",IF(H74-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N74" s="51" t="n"/>
@@ -6482,7 +6517,7 @@
         <v/>
       </c>
       <c r="M75" s="58">
-        <f>IF(B75="","",IF(E75="Done","✓ Done",IF(E75="Blocked","Blocked",IF(H75="","No due date",IF(H75&lt;NOW(),"Overdue",IF(H75-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B75="","",IF(E75="Done","Complete",IF(E75="Blocked","Blocked",IF(H75="","No due date",IF(H75&lt;NOW(),"Overdue",IF(H75-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N75" s="51" t="n"/>
@@ -6512,7 +6547,7 @@
         <v/>
       </c>
       <c r="M76" s="58">
-        <f>IF(B76="","",IF(E76="Done","✓ Done",IF(E76="Blocked","Blocked",IF(H76="","No due date",IF(H76&lt;NOW(),"Overdue",IF(H76-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B76="","",IF(E76="Done","Complete",IF(E76="Blocked","Blocked",IF(H76="","No due date",IF(H76&lt;NOW(),"Overdue",IF(H76-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N76" s="51" t="n"/>
@@ -6542,7 +6577,7 @@
         <v/>
       </c>
       <c r="M77" s="58">
-        <f>IF(B77="","",IF(E77="Done","✓ Done",IF(E77="Blocked","Blocked",IF(H77="","No due date",IF(H77&lt;NOW(),"Overdue",IF(H77-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B77="","",IF(E77="Done","Complete",IF(E77="Blocked","Blocked",IF(H77="","No due date",IF(H77&lt;NOW(),"Overdue",IF(H77-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N77" s="51" t="n"/>
@@ -6572,7 +6607,7 @@
         <v/>
       </c>
       <c r="M78" s="58">
-        <f>IF(B78="","",IF(E78="Done","✓ Done",IF(E78="Blocked","Blocked",IF(H78="","No due date",IF(H78&lt;NOW(),"Overdue",IF(H78-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B78="","",IF(E78="Done","Complete",IF(E78="Blocked","Blocked",IF(H78="","No due date",IF(H78&lt;NOW(),"Overdue",IF(H78-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N78" s="51" t="n"/>
@@ -6602,7 +6637,7 @@
         <v/>
       </c>
       <c r="M79" s="58">
-        <f>IF(B79="","",IF(E79="Done","✓ Done",IF(E79="Blocked","Blocked",IF(H79="","No due date",IF(H79&lt;NOW(),"Overdue",IF(H79-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B79="","",IF(E79="Done","Complete",IF(E79="Blocked","Blocked",IF(H79="","No due date",IF(H79&lt;NOW(),"Overdue",IF(H79-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N79" s="51" t="n"/>
@@ -6632,7 +6667,7 @@
         <v/>
       </c>
       <c r="M80" s="58">
-        <f>IF(B80="","",IF(E80="Done","✓ Done",IF(E80="Blocked","Blocked",IF(H80="","No due date",IF(H80&lt;NOW(),"Overdue",IF(H80-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B80="","",IF(E80="Done","Complete",IF(E80="Blocked","Blocked",IF(H80="","No due date",IF(H80&lt;NOW(),"Overdue",IF(H80-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N80" s="51" t="n"/>
@@ -6662,7 +6697,7 @@
         <v/>
       </c>
       <c r="M81" s="58">
-        <f>IF(B81="","",IF(E81="Done","✓ Done",IF(E81="Blocked","Blocked",IF(H81="","No due date",IF(H81&lt;NOW(),"Overdue",IF(H81-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B81="","",IF(E81="Done","Complete",IF(E81="Blocked","Blocked",IF(H81="","No due date",IF(H81&lt;NOW(),"Overdue",IF(H81-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N81" s="51" t="n"/>
@@ -6692,7 +6727,7 @@
         <v/>
       </c>
       <c r="M82" s="58">
-        <f>IF(B82="","",IF(E82="Done","✓ Done",IF(E82="Blocked","Blocked",IF(H82="","No due date",IF(H82&lt;NOW(),"Overdue",IF(H82-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B82="","",IF(E82="Done","Complete",IF(E82="Blocked","Blocked",IF(H82="","No due date",IF(H82&lt;NOW(),"Overdue",IF(H82-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N82" s="51" t="n"/>
@@ -6722,7 +6757,7 @@
         <v/>
       </c>
       <c r="M83" s="58">
-        <f>IF(B83="","",IF(E83="Done","✓ Done",IF(E83="Blocked","Blocked",IF(H83="","No due date",IF(H83&lt;NOW(),"Overdue",IF(H83-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B83="","",IF(E83="Done","Complete",IF(E83="Blocked","Blocked",IF(H83="","No due date",IF(H83&lt;NOW(),"Overdue",IF(H83-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N83" s="51" t="n"/>
@@ -6752,7 +6787,7 @@
         <v/>
       </c>
       <c r="M84" s="58">
-        <f>IF(B84="","",IF(E84="Done","✓ Done",IF(E84="Blocked","Blocked",IF(H84="","No due date",IF(H84&lt;NOW(),"Overdue",IF(H84-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B84="","",IF(E84="Done","Complete",IF(E84="Blocked","Blocked",IF(H84="","No due date",IF(H84&lt;NOW(),"Overdue",IF(H84-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N84" s="51" t="n"/>
@@ -6782,7 +6817,7 @@
         <v/>
       </c>
       <c r="M85" s="58">
-        <f>IF(B85="","",IF(E85="Done","✓ Done",IF(E85="Blocked","Blocked",IF(H85="","No due date",IF(H85&lt;NOW(),"Overdue",IF(H85-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B85="","",IF(E85="Done","Complete",IF(E85="Blocked","Blocked",IF(H85="","No due date",IF(H85&lt;NOW(),"Overdue",IF(H85-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N85" s="51" t="n"/>
@@ -6812,7 +6847,7 @@
         <v/>
       </c>
       <c r="M86" s="58">
-        <f>IF(B86="","",IF(E86="Done","✓ Done",IF(E86="Blocked","Blocked",IF(H86="","No due date",IF(H86&lt;NOW(),"Overdue",IF(H86-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B86="","",IF(E86="Done","Complete",IF(E86="Blocked","Blocked",IF(H86="","No due date",IF(H86&lt;NOW(),"Overdue",IF(H86-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N86" s="51" t="n"/>
@@ -6842,7 +6877,7 @@
         <v/>
       </c>
       <c r="M87" s="58">
-        <f>IF(B87="","",IF(E87="Done","✓ Done",IF(E87="Blocked","Blocked",IF(H87="","No due date",IF(H87&lt;NOW(),"Overdue",IF(H87-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B87="","",IF(E87="Done","Complete",IF(E87="Blocked","Blocked",IF(H87="","No due date",IF(H87&lt;NOW(),"Overdue",IF(H87-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N87" s="51" t="n"/>
@@ -6872,7 +6907,7 @@
         <v/>
       </c>
       <c r="M88" s="58">
-        <f>IF(B88="","",IF(E88="Done","✓ Done",IF(E88="Blocked","Blocked",IF(H88="","No due date",IF(H88&lt;NOW(),"Overdue",IF(H88-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B88="","",IF(E88="Done","Complete",IF(E88="Blocked","Blocked",IF(H88="","No due date",IF(H88&lt;NOW(),"Overdue",IF(H88-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N88" s="51" t="n"/>
@@ -6902,7 +6937,7 @@
         <v/>
       </c>
       <c r="M89" s="58">
-        <f>IF(B89="","",IF(E89="Done","✓ Done",IF(E89="Blocked","Blocked",IF(H89="","No due date",IF(H89&lt;NOW(),"Overdue",IF(H89-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B89="","",IF(E89="Done","Complete",IF(E89="Blocked","Blocked",IF(H89="","No due date",IF(H89&lt;NOW(),"Overdue",IF(H89-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N89" s="51" t="n"/>
@@ -6932,7 +6967,7 @@
         <v/>
       </c>
       <c r="M90" s="58">
-        <f>IF(B90="","",IF(E90="Done","✓ Done",IF(E90="Blocked","Blocked",IF(H90="","No due date",IF(H90&lt;NOW(),"Overdue",IF(H90-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B90="","",IF(E90="Done","Complete",IF(E90="Blocked","Blocked",IF(H90="","No due date",IF(H90&lt;NOW(),"Overdue",IF(H90-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N90" s="51" t="n"/>
@@ -6962,7 +6997,7 @@
         <v/>
       </c>
       <c r="M91" s="58">
-        <f>IF(B91="","",IF(E91="Done","✓ Done",IF(E91="Blocked","Blocked",IF(H91="","No due date",IF(H91&lt;NOW(),"Overdue",IF(H91-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B91="","",IF(E91="Done","Complete",IF(E91="Blocked","Blocked",IF(H91="","No due date",IF(H91&lt;NOW(),"Overdue",IF(H91-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N91" s="51" t="n"/>
@@ -6992,7 +7027,7 @@
         <v/>
       </c>
       <c r="M92" s="58">
-        <f>IF(B92="","",IF(E92="Done","✓ Done",IF(E92="Blocked","Blocked",IF(H92="","No due date",IF(H92&lt;NOW(),"Overdue",IF(H92-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B92="","",IF(E92="Done","Complete",IF(E92="Blocked","Blocked",IF(H92="","No due date",IF(H92&lt;NOW(),"Overdue",IF(H92-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N92" s="51" t="n"/>
@@ -7022,7 +7057,7 @@
         <v/>
       </c>
       <c r="M93" s="58">
-        <f>IF(B93="","",IF(E93="Done","✓ Done",IF(E93="Blocked","Blocked",IF(H93="","No due date",IF(H93&lt;NOW(),"Overdue",IF(H93-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B93="","",IF(E93="Done","Complete",IF(E93="Blocked","Blocked",IF(H93="","No due date",IF(H93&lt;NOW(),"Overdue",IF(H93-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N93" s="51" t="n"/>
@@ -7052,7 +7087,7 @@
         <v/>
       </c>
       <c r="M94" s="58">
-        <f>IF(B94="","",IF(E94="Done","✓ Done",IF(E94="Blocked","Blocked",IF(H94="","No due date",IF(H94&lt;NOW(),"Overdue",IF(H94-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B94="","",IF(E94="Done","Complete",IF(E94="Blocked","Blocked",IF(H94="","No due date",IF(H94&lt;NOW(),"Overdue",IF(H94-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N94" s="51" t="n"/>
@@ -7082,7 +7117,7 @@
         <v/>
       </c>
       <c r="M95" s="58">
-        <f>IF(B95="","",IF(E95="Done","✓ Done",IF(E95="Blocked","Blocked",IF(H95="","No due date",IF(H95&lt;NOW(),"Overdue",IF(H95-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B95="","",IF(E95="Done","Complete",IF(E95="Blocked","Blocked",IF(H95="","No due date",IF(H95&lt;NOW(),"Overdue",IF(H95-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N95" s="51" t="n"/>
@@ -7112,7 +7147,7 @@
         <v/>
       </c>
       <c r="M96" s="58">
-        <f>IF(B96="","",IF(E96="Done","✓ Done",IF(E96="Blocked","Blocked",IF(H96="","No due date",IF(H96&lt;NOW(),"Overdue",IF(H96-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B96="","",IF(E96="Done","Complete",IF(E96="Blocked","Blocked",IF(H96="","No due date",IF(H96&lt;NOW(),"Overdue",IF(H96-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N96" s="51" t="n"/>
@@ -7142,7 +7177,7 @@
         <v/>
       </c>
       <c r="M97" s="58">
-        <f>IF(B97="","",IF(E97="Done","✓ Done",IF(E97="Blocked","Blocked",IF(H97="","No due date",IF(H97&lt;NOW(),"Overdue",IF(H97-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B97="","",IF(E97="Done","Complete",IF(E97="Blocked","Blocked",IF(H97="","No due date",IF(H97&lt;NOW(),"Overdue",IF(H97-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N97" s="51" t="n"/>
@@ -7172,7 +7207,7 @@
         <v/>
       </c>
       <c r="M98" s="58">
-        <f>IF(B98="","",IF(E98="Done","✓ Done",IF(E98="Blocked","Blocked",IF(H98="","No due date",IF(H98&lt;NOW(),"Overdue",IF(H98-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B98="","",IF(E98="Done","Complete",IF(E98="Blocked","Blocked",IF(H98="","No due date",IF(H98&lt;NOW(),"Overdue",IF(H98-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N98" s="51" t="n"/>
@@ -7202,7 +7237,7 @@
         <v/>
       </c>
       <c r="M99" s="58">
-        <f>IF(B99="","",IF(E99="Done","✓ Done",IF(E99="Blocked","Blocked",IF(H99="","No due date",IF(H99&lt;NOW(),"Overdue",IF(H99-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B99="","",IF(E99="Done","Complete",IF(E99="Blocked","Blocked",IF(H99="","No due date",IF(H99&lt;NOW(),"Overdue",IF(H99-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N99" s="51" t="n"/>
@@ -7232,7 +7267,7 @@
         <v/>
       </c>
       <c r="M100" s="58">
-        <f>IF(B100="","",IF(E100="Done","✓ Done",IF(E100="Blocked","Blocked",IF(H100="","No due date",IF(H100&lt;NOW(),"Overdue",IF(H100-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B100="","",IF(E100="Done","Complete",IF(E100="Blocked","Blocked",IF(H100="","No due date",IF(H100&lt;NOW(),"Overdue",IF(H100-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N100" s="51" t="n"/>
@@ -7262,7 +7297,7 @@
         <v/>
       </c>
       <c r="M101" s="58">
-        <f>IF(B101="","",IF(E101="Done","✓ Done",IF(E101="Blocked","Blocked",IF(H101="","No due date",IF(H101&lt;NOW(),"Overdue",IF(H101-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B101="","",IF(E101="Done","Complete",IF(E101="Blocked","Blocked",IF(H101="","No due date",IF(H101&lt;NOW(),"Overdue",IF(H101-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N101" s="51" t="n"/>
@@ -7292,7 +7327,7 @@
         <v/>
       </c>
       <c r="M102" s="58">
-        <f>IF(B102="","",IF(E102="Done","✓ Done",IF(E102="Blocked","Blocked",IF(H102="","No due date",IF(H102&lt;NOW(),"Overdue",IF(H102-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B102="","",IF(E102="Done","Complete",IF(E102="Blocked","Blocked",IF(H102="","No due date",IF(H102&lt;NOW(),"Overdue",IF(H102-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N102" s="51" t="n"/>
@@ -7322,7 +7357,7 @@
         <v/>
       </c>
       <c r="M103" s="58">
-        <f>IF(B103="","",IF(E103="Done","✓ Done",IF(E103="Blocked","Blocked",IF(H103="","No due date",IF(H103&lt;NOW(),"Overdue",IF(H103-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B103="","",IF(E103="Done","Complete",IF(E103="Blocked","Blocked",IF(H103="","No due date",IF(H103&lt;NOW(),"Overdue",IF(H103-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N103" s="51" t="n"/>
@@ -7352,7 +7387,7 @@
         <v/>
       </c>
       <c r="M104" s="58">
-        <f>IF(B104="","",IF(E104="Done","✓ Done",IF(E104="Blocked","Blocked",IF(H104="","No due date",IF(H104&lt;NOW(),"Overdue",IF(H104-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B104="","",IF(E104="Done","Complete",IF(E104="Blocked","Blocked",IF(H104="","No due date",IF(H104&lt;NOW(),"Overdue",IF(H104-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N104" s="51" t="n"/>
@@ -7382,7 +7417,7 @@
         <v/>
       </c>
       <c r="M105" s="58">
-        <f>IF(B105="","",IF(E105="Done","✓ Done",IF(E105="Blocked","Blocked",IF(H105="","No due date",IF(H105&lt;NOW(),"Overdue",IF(H105-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B105="","",IF(E105="Done","Complete",IF(E105="Blocked","Blocked",IF(H105="","No due date",IF(H105&lt;NOW(),"Overdue",IF(H105-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N105" s="51" t="n"/>
@@ -7412,7 +7447,7 @@
         <v/>
       </c>
       <c r="M106" s="58">
-        <f>IF(B106="","",IF(E106="Done","✓ Done",IF(E106="Blocked","Blocked",IF(H106="","No due date",IF(H106&lt;NOW(),"Overdue",IF(H106-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B106="","",IF(E106="Done","Complete",IF(E106="Blocked","Blocked",IF(H106="","No due date",IF(H106&lt;NOW(),"Overdue",IF(H106-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N106" s="51" t="n"/>
@@ -7442,7 +7477,7 @@
         <v/>
       </c>
       <c r="M107" s="58">
-        <f>IF(B107="","",IF(E107="Done","✓ Done",IF(E107="Blocked","Blocked",IF(H107="","No due date",IF(H107&lt;NOW(),"Overdue",IF(H107-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B107="","",IF(E107="Done","Complete",IF(E107="Blocked","Blocked",IF(H107="","No due date",IF(H107&lt;NOW(),"Overdue",IF(H107-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N107" s="51" t="n"/>
@@ -7472,7 +7507,7 @@
         <v/>
       </c>
       <c r="M108" s="58">
-        <f>IF(B108="","",IF(E108="Done","✓ Done",IF(E108="Blocked","Blocked",IF(H108="","No due date",IF(H108&lt;NOW(),"Overdue",IF(H108-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B108="","",IF(E108="Done","Complete",IF(E108="Blocked","Blocked",IF(H108="","No due date",IF(H108&lt;NOW(),"Overdue",IF(H108-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N108" s="51" t="n"/>
@@ -7502,7 +7537,7 @@
         <v/>
       </c>
       <c r="M109" s="58">
-        <f>IF(B109="","",IF(E109="Done","✓ Done",IF(E109="Blocked","Blocked",IF(H109="","No due date",IF(H109&lt;NOW(),"Overdue",IF(H109-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B109="","",IF(E109="Done","Complete",IF(E109="Blocked","Blocked",IF(H109="","No due date",IF(H109&lt;NOW(),"Overdue",IF(H109-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N109" s="51" t="n"/>
@@ -7532,7 +7567,7 @@
         <v/>
       </c>
       <c r="M110" s="58">
-        <f>IF(B110="","",IF(E110="Done","✓ Done",IF(E110="Blocked","Blocked",IF(H110="","No due date",IF(H110&lt;NOW(),"Overdue",IF(H110-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B110="","",IF(E110="Done","Complete",IF(E110="Blocked","Blocked",IF(H110="","No due date",IF(H110&lt;NOW(),"Overdue",IF(H110-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N110" s="51" t="n"/>
@@ -7562,7 +7597,7 @@
         <v/>
       </c>
       <c r="M111" s="58">
-        <f>IF(B111="","",IF(E111="Done","✓ Done",IF(E111="Blocked","Blocked",IF(H111="","No due date",IF(H111&lt;NOW(),"Overdue",IF(H111-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B111="","",IF(E111="Done","Complete",IF(E111="Blocked","Blocked",IF(H111="","No due date",IF(H111&lt;NOW(),"Overdue",IF(H111-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N111" s="51" t="n"/>
@@ -7592,7 +7627,7 @@
         <v/>
       </c>
       <c r="M112" s="58">
-        <f>IF(B112="","",IF(E112="Done","✓ Done",IF(E112="Blocked","Blocked",IF(H112="","No due date",IF(H112&lt;NOW(),"Overdue",IF(H112-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B112="","",IF(E112="Done","Complete",IF(E112="Blocked","Blocked",IF(H112="","No due date",IF(H112&lt;NOW(),"Overdue",IF(H112-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N112" s="51" t="n"/>
@@ -7622,7 +7657,7 @@
         <v/>
       </c>
       <c r="M113" s="58">
-        <f>IF(B113="","",IF(E113="Done","✓ Done",IF(E113="Blocked","Blocked",IF(H113="","No due date",IF(H113&lt;NOW(),"Overdue",IF(H113-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B113="","",IF(E113="Done","Complete",IF(E113="Blocked","Blocked",IF(H113="","No due date",IF(H113&lt;NOW(),"Overdue",IF(H113-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N113" s="51" t="n"/>
@@ -7652,7 +7687,7 @@
         <v/>
       </c>
       <c r="M114" s="58">
-        <f>IF(B114="","",IF(E114="Done","✓ Done",IF(E114="Blocked","Blocked",IF(H114="","No due date",IF(H114&lt;NOW(),"Overdue",IF(H114-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B114="","",IF(E114="Done","Complete",IF(E114="Blocked","Blocked",IF(H114="","No due date",IF(H114&lt;NOW(),"Overdue",IF(H114-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N114" s="51" t="n"/>
@@ -7682,7 +7717,7 @@
         <v/>
       </c>
       <c r="M115" s="58">
-        <f>IF(B115="","",IF(E115="Done","✓ Done",IF(E115="Blocked","Blocked",IF(H115="","No due date",IF(H115&lt;NOW(),"Overdue",IF(H115-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B115="","",IF(E115="Done","Complete",IF(E115="Blocked","Blocked",IF(H115="","No due date",IF(H115&lt;NOW(),"Overdue",IF(H115-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N115" s="51" t="n"/>
@@ -7712,7 +7747,7 @@
         <v/>
       </c>
       <c r="M116" s="58">
-        <f>IF(B116="","",IF(E116="Done","✓ Done",IF(E116="Blocked","Blocked",IF(H116="","No due date",IF(H116&lt;NOW(),"Overdue",IF(H116-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B116="","",IF(E116="Done","Complete",IF(E116="Blocked","Blocked",IF(H116="","No due date",IF(H116&lt;NOW(),"Overdue",IF(H116-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N116" s="51" t="n"/>
@@ -7742,7 +7777,7 @@
         <v/>
       </c>
       <c r="M117" s="58">
-        <f>IF(B117="","",IF(E117="Done","✓ Done",IF(E117="Blocked","Blocked",IF(H117="","No due date",IF(H117&lt;NOW(),"Overdue",IF(H117-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B117="","",IF(E117="Done","Complete",IF(E117="Blocked","Blocked",IF(H117="","No due date",IF(H117&lt;NOW(),"Overdue",IF(H117-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N117" s="51" t="n"/>
@@ -7772,7 +7807,7 @@
         <v/>
       </c>
       <c r="M118" s="58">
-        <f>IF(B118="","",IF(E118="Done","✓ Done",IF(E118="Blocked","Blocked",IF(H118="","No due date",IF(H118&lt;NOW(),"Overdue",IF(H118-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B118="","",IF(E118="Done","Complete",IF(E118="Blocked","Blocked",IF(H118="","No due date",IF(H118&lt;NOW(),"Overdue",IF(H118-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N118" s="51" t="n"/>
@@ -7802,7 +7837,7 @@
         <v/>
       </c>
       <c r="M119" s="58">
-        <f>IF(B119="","",IF(E119="Done","✓ Done",IF(E119="Blocked","Blocked",IF(H119="","No due date",IF(H119&lt;NOW(),"Overdue",IF(H119-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B119="","",IF(E119="Done","Complete",IF(E119="Blocked","Blocked",IF(H119="","No due date",IF(H119&lt;NOW(),"Overdue",IF(H119-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N119" s="51" t="n"/>
@@ -7832,7 +7867,7 @@
         <v/>
       </c>
       <c r="M120" s="58">
-        <f>IF(B120="","",IF(E120="Done","✓ Done",IF(E120="Blocked","Blocked",IF(H120="","No due date",IF(H120&lt;NOW(),"Overdue",IF(H120-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B120="","",IF(E120="Done","Complete",IF(E120="Blocked","Blocked",IF(H120="","No due date",IF(H120&lt;NOW(),"Overdue",IF(H120-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N120" s="51" t="n"/>
@@ -7862,7 +7897,7 @@
         <v/>
       </c>
       <c r="M121" s="58">
-        <f>IF(B121="","",IF(E121="Done","✓ Done",IF(E121="Blocked","Blocked",IF(H121="","No due date",IF(H121&lt;NOW(),"Overdue",IF(H121-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B121="","",IF(E121="Done","Complete",IF(E121="Blocked","Blocked",IF(H121="","No due date",IF(H121&lt;NOW(),"Overdue",IF(H121-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N121" s="51" t="n"/>
@@ -7892,7 +7927,7 @@
         <v/>
       </c>
       <c r="M122" s="58">
-        <f>IF(B122="","",IF(E122="Done","✓ Done",IF(E122="Blocked","Blocked",IF(H122="","No due date",IF(H122&lt;NOW(),"Overdue",IF(H122-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B122="","",IF(E122="Done","Complete",IF(E122="Blocked","Blocked",IF(H122="","No due date",IF(H122&lt;NOW(),"Overdue",IF(H122-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N122" s="51" t="n"/>
@@ -7922,7 +7957,7 @@
         <v/>
       </c>
       <c r="M123" s="58">
-        <f>IF(B123="","",IF(E123="Done","✓ Done",IF(E123="Blocked","Blocked",IF(H123="","No due date",IF(H123&lt;NOW(),"Overdue",IF(H123-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B123="","",IF(E123="Done","Complete",IF(E123="Blocked","Blocked",IF(H123="","No due date",IF(H123&lt;NOW(),"Overdue",IF(H123-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N123" s="51" t="n"/>
@@ -7952,7 +7987,7 @@
         <v/>
       </c>
       <c r="M124" s="58">
-        <f>IF(B124="","",IF(E124="Done","✓ Done",IF(E124="Blocked","Blocked",IF(H124="","No due date",IF(H124&lt;NOW(),"Overdue",IF(H124-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B124="","",IF(E124="Done","Complete",IF(E124="Blocked","Blocked",IF(H124="","No due date",IF(H124&lt;NOW(),"Overdue",IF(H124-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N124" s="51" t="n"/>
@@ -7982,7 +8017,7 @@
         <v/>
       </c>
       <c r="M125" s="58">
-        <f>IF(B125="","",IF(E125="Done","✓ Done",IF(E125="Blocked","Blocked",IF(H125="","No due date",IF(H125&lt;NOW(),"Overdue",IF(H125-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B125="","",IF(E125="Done","Complete",IF(E125="Blocked","Blocked",IF(H125="","No due date",IF(H125&lt;NOW(),"Overdue",IF(H125-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N125" s="51" t="n"/>
@@ -8012,7 +8047,7 @@
         <v/>
       </c>
       <c r="M126" s="58">
-        <f>IF(B126="","",IF(E126="Done","✓ Done",IF(E126="Blocked","Blocked",IF(H126="","No due date",IF(H126&lt;NOW(),"Overdue",IF(H126-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B126="","",IF(E126="Done","Complete",IF(E126="Blocked","Blocked",IF(H126="","No due date",IF(H126&lt;NOW(),"Overdue",IF(H126-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N126" s="51" t="n"/>
@@ -8042,7 +8077,7 @@
         <v/>
       </c>
       <c r="M127" s="58">
-        <f>IF(B127="","",IF(E127="Done","✓ Done",IF(E127="Blocked","Blocked",IF(H127="","No due date",IF(H127&lt;NOW(),"Overdue",IF(H127-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B127="","",IF(E127="Done","Complete",IF(E127="Blocked","Blocked",IF(H127="","No due date",IF(H127&lt;NOW(),"Overdue",IF(H127-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N127" s="51" t="n"/>
@@ -8072,7 +8107,7 @@
         <v/>
       </c>
       <c r="M128" s="58">
-        <f>IF(B128="","",IF(E128="Done","✓ Done",IF(E128="Blocked","Blocked",IF(H128="","No due date",IF(H128&lt;NOW(),"Overdue",IF(H128-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B128="","",IF(E128="Done","Complete",IF(E128="Blocked","Blocked",IF(H128="","No due date",IF(H128&lt;NOW(),"Overdue",IF(H128-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N128" s="51" t="n"/>
@@ -8102,7 +8137,7 @@
         <v/>
       </c>
       <c r="M129" s="58">
-        <f>IF(B129="","",IF(E129="Done","✓ Done",IF(E129="Blocked","Blocked",IF(H129="","No due date",IF(H129&lt;NOW(),"Overdue",IF(H129-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B129="","",IF(E129="Done","Complete",IF(E129="Blocked","Blocked",IF(H129="","No due date",IF(H129&lt;NOW(),"Overdue",IF(H129-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N129" s="51" t="n"/>
@@ -8132,7 +8167,7 @@
         <v/>
       </c>
       <c r="M130" s="58">
-        <f>IF(B130="","",IF(E130="Done","✓ Done",IF(E130="Blocked","Blocked",IF(H130="","No due date",IF(H130&lt;NOW(),"Overdue",IF(H130-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B130="","",IF(E130="Done","Complete",IF(E130="Blocked","Blocked",IF(H130="","No due date",IF(H130&lt;NOW(),"Overdue",IF(H130-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N130" s="51" t="n"/>
@@ -8162,7 +8197,7 @@
         <v/>
       </c>
       <c r="M131" s="58">
-        <f>IF(B131="","",IF(E131="Done","✓ Done",IF(E131="Blocked","Blocked",IF(H131="","No due date",IF(H131&lt;NOW(),"Overdue",IF(H131-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B131="","",IF(E131="Done","Complete",IF(E131="Blocked","Blocked",IF(H131="","No due date",IF(H131&lt;NOW(),"Overdue",IF(H131-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N131" s="51" t="n"/>
@@ -8192,7 +8227,7 @@
         <v/>
       </c>
       <c r="M132" s="58">
-        <f>IF(B132="","",IF(E132="Done","✓ Done",IF(E132="Blocked","Blocked",IF(H132="","No due date",IF(H132&lt;NOW(),"Overdue",IF(H132-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B132="","",IF(E132="Done","Complete",IF(E132="Blocked","Blocked",IF(H132="","No due date",IF(H132&lt;NOW(),"Overdue",IF(H132-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N132" s="51" t="n"/>
@@ -8222,7 +8257,7 @@
         <v/>
       </c>
       <c r="M133" s="58">
-        <f>IF(B133="","",IF(E133="Done","✓ Done",IF(E133="Blocked","Blocked",IF(H133="","No due date",IF(H133&lt;NOW(),"Overdue",IF(H133-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B133="","",IF(E133="Done","Complete",IF(E133="Blocked","Blocked",IF(H133="","No due date",IF(H133&lt;NOW(),"Overdue",IF(H133-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N133" s="51" t="n"/>
@@ -8252,7 +8287,7 @@
         <v/>
       </c>
       <c r="M134" s="58">
-        <f>IF(B134="","",IF(E134="Done","✓ Done",IF(E134="Blocked","Blocked",IF(H134="","No due date",IF(H134&lt;NOW(),"Overdue",IF(H134-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B134="","",IF(E134="Done","Complete",IF(E134="Blocked","Blocked",IF(H134="","No due date",IF(H134&lt;NOW(),"Overdue",IF(H134-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N134" s="51" t="n"/>
@@ -8282,7 +8317,7 @@
         <v/>
       </c>
       <c r="M135" s="58">
-        <f>IF(B135="","",IF(E135="Done","✓ Done",IF(E135="Blocked","Blocked",IF(H135="","No due date",IF(H135&lt;NOW(),"Overdue",IF(H135-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B135="","",IF(E135="Done","Complete",IF(E135="Blocked","Blocked",IF(H135="","No due date",IF(H135&lt;NOW(),"Overdue",IF(H135-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N135" s="51" t="n"/>
@@ -8312,7 +8347,7 @@
         <v/>
       </c>
       <c r="M136" s="58">
-        <f>IF(B136="","",IF(E136="Done","✓ Done",IF(E136="Blocked","Blocked",IF(H136="","No due date",IF(H136&lt;NOW(),"Overdue",IF(H136-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B136="","",IF(E136="Done","Complete",IF(E136="Blocked","Blocked",IF(H136="","No due date",IF(H136&lt;NOW(),"Overdue",IF(H136-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N136" s="51" t="n"/>
@@ -8342,7 +8377,7 @@
         <v/>
       </c>
       <c r="M137" s="58">
-        <f>IF(B137="","",IF(E137="Done","✓ Done",IF(E137="Blocked","Blocked",IF(H137="","No due date",IF(H137&lt;NOW(),"Overdue",IF(H137-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B137="","",IF(E137="Done","Complete",IF(E137="Blocked","Blocked",IF(H137="","No due date",IF(H137&lt;NOW(),"Overdue",IF(H137-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N137" s="51" t="n"/>
@@ -8372,7 +8407,7 @@
         <v/>
       </c>
       <c r="M138" s="58">
-        <f>IF(B138="","",IF(E138="Done","✓ Done",IF(E138="Blocked","Blocked",IF(H138="","No due date",IF(H138&lt;NOW(),"Overdue",IF(H138-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B138="","",IF(E138="Done","Complete",IF(E138="Blocked","Blocked",IF(H138="","No due date",IF(H138&lt;NOW(),"Overdue",IF(H138-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N138" s="51" t="n"/>
@@ -8402,7 +8437,7 @@
         <v/>
       </c>
       <c r="M139" s="58">
-        <f>IF(B139="","",IF(E139="Done","✓ Done",IF(E139="Blocked","Blocked",IF(H139="","No due date",IF(H139&lt;NOW(),"Overdue",IF(H139-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B139="","",IF(E139="Done","Complete",IF(E139="Blocked","Blocked",IF(H139="","No due date",IF(H139&lt;NOW(),"Overdue",IF(H139-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N139" s="51" t="n"/>
@@ -8432,7 +8467,7 @@
         <v/>
       </c>
       <c r="M140" s="58">
-        <f>IF(B140="","",IF(E140="Done","✓ Done",IF(E140="Blocked","Blocked",IF(H140="","No due date",IF(H140&lt;NOW(),"Overdue",IF(H140-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B140="","",IF(E140="Done","Complete",IF(E140="Blocked","Blocked",IF(H140="","No due date",IF(H140&lt;NOW(),"Overdue",IF(H140-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N140" s="51" t="n"/>
@@ -8462,7 +8497,7 @@
         <v/>
       </c>
       <c r="M141" s="58">
-        <f>IF(B141="","",IF(E141="Done","✓ Done",IF(E141="Blocked","Blocked",IF(H141="","No due date",IF(H141&lt;NOW(),"Overdue",IF(H141-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B141="","",IF(E141="Done","Complete",IF(E141="Blocked","Blocked",IF(H141="","No due date",IF(H141&lt;NOW(),"Overdue",IF(H141-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N141" s="51" t="n"/>
@@ -8492,7 +8527,7 @@
         <v/>
       </c>
       <c r="M142" s="58">
-        <f>IF(B142="","",IF(E142="Done","✓ Done",IF(E142="Blocked","Blocked",IF(H142="","No due date",IF(H142&lt;NOW(),"Overdue",IF(H142-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B142="","",IF(E142="Done","Complete",IF(E142="Blocked","Blocked",IF(H142="","No due date",IF(H142&lt;NOW(),"Overdue",IF(H142-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N142" s="51" t="n"/>
@@ -8522,7 +8557,7 @@
         <v/>
       </c>
       <c r="M143" s="58">
-        <f>IF(B143="","",IF(E143="Done","✓ Done",IF(E143="Blocked","Blocked",IF(H143="","No due date",IF(H143&lt;NOW(),"Overdue",IF(H143-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B143="","",IF(E143="Done","Complete",IF(E143="Blocked","Blocked",IF(H143="","No due date",IF(H143&lt;NOW(),"Overdue",IF(H143-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N143" s="51" t="n"/>
@@ -8552,7 +8587,7 @@
         <v/>
       </c>
       <c r="M144" s="58">
-        <f>IF(B144="","",IF(E144="Done","✓ Done",IF(E144="Blocked","Blocked",IF(H144="","No due date",IF(H144&lt;NOW(),"Overdue",IF(H144-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B144="","",IF(E144="Done","Complete",IF(E144="Blocked","Blocked",IF(H144="","No due date",IF(H144&lt;NOW(),"Overdue",IF(H144-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N144" s="51" t="n"/>
@@ -8582,7 +8617,7 @@
         <v/>
       </c>
       <c r="M145" s="58">
-        <f>IF(B145="","",IF(E145="Done","✓ Done",IF(E145="Blocked","Blocked",IF(H145="","No due date",IF(H145&lt;NOW(),"Overdue",IF(H145-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B145="","",IF(E145="Done","Complete",IF(E145="Blocked","Blocked",IF(H145="","No due date",IF(H145&lt;NOW(),"Overdue",IF(H145-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N145" s="51" t="n"/>
@@ -8612,7 +8647,7 @@
         <v/>
       </c>
       <c r="M146" s="58">
-        <f>IF(B146="","",IF(E146="Done","✓ Done",IF(E146="Blocked","Blocked",IF(H146="","No due date",IF(H146&lt;NOW(),"Overdue",IF(H146-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B146="","",IF(E146="Done","Complete",IF(E146="Blocked","Blocked",IF(H146="","No due date",IF(H146&lt;NOW(),"Overdue",IF(H146-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N146" s="51" t="n"/>
@@ -8642,7 +8677,7 @@
         <v/>
       </c>
       <c r="M147" s="58">
-        <f>IF(B147="","",IF(E147="Done","✓ Done",IF(E147="Blocked","Blocked",IF(H147="","No due date",IF(H147&lt;NOW(),"Overdue",IF(H147-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B147="","",IF(E147="Done","Complete",IF(E147="Blocked","Blocked",IF(H147="","No due date",IF(H147&lt;NOW(),"Overdue",IF(H147-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N147" s="51" t="n"/>
@@ -8672,7 +8707,7 @@
         <v/>
       </c>
       <c r="M148" s="58">
-        <f>IF(B148="","",IF(E148="Done","✓ Done",IF(E148="Blocked","Blocked",IF(H148="","No due date",IF(H148&lt;NOW(),"Overdue",IF(H148-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B148="","",IF(E148="Done","Complete",IF(E148="Blocked","Blocked",IF(H148="","No due date",IF(H148&lt;NOW(),"Overdue",IF(H148-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N148" s="51" t="n"/>
@@ -8702,7 +8737,7 @@
         <v/>
       </c>
       <c r="M149" s="58">
-        <f>IF(B149="","",IF(E149="Done","✓ Done",IF(E149="Blocked","Blocked",IF(H149="","No due date",IF(H149&lt;NOW(),"Overdue",IF(H149-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B149="","",IF(E149="Done","Complete",IF(E149="Blocked","Blocked",IF(H149="","No due date",IF(H149&lt;NOW(),"Overdue",IF(H149-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N149" s="51" t="n"/>
@@ -8732,7 +8767,7 @@
         <v/>
       </c>
       <c r="M150" s="58">
-        <f>IF(B150="","",IF(E150="Done","✓ Done",IF(E150="Blocked","Blocked",IF(H150="","No due date",IF(H150&lt;NOW(),"Overdue",IF(H150-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B150="","",IF(E150="Done","Complete",IF(E150="Blocked","Blocked",IF(H150="","No due date",IF(H150&lt;NOW(),"Overdue",IF(H150-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N150" s="51" t="n"/>
@@ -8762,7 +8797,7 @@
         <v/>
       </c>
       <c r="M151" s="58">
-        <f>IF(B151="","",IF(E151="Done","✓ Done",IF(E151="Blocked","Blocked",IF(H151="","No due date",IF(H151&lt;NOW(),"Overdue",IF(H151-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B151="","",IF(E151="Done","Complete",IF(E151="Blocked","Blocked",IF(H151="","No due date",IF(H151&lt;NOW(),"Overdue",IF(H151-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N151" s="51" t="n"/>
@@ -8792,7 +8827,7 @@
         <v/>
       </c>
       <c r="M152" s="58">
-        <f>IF(B152="","",IF(E152="Done","✓ Done",IF(E152="Blocked","Blocked",IF(H152="","No due date",IF(H152&lt;NOW(),"Overdue",IF(H152-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B152="","",IF(E152="Done","Complete",IF(E152="Blocked","Blocked",IF(H152="","No due date",IF(H152&lt;NOW(),"Overdue",IF(H152-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N152" s="51" t="n"/>
@@ -8822,7 +8857,7 @@
         <v/>
       </c>
       <c r="M153" s="58">
-        <f>IF(B153="","",IF(E153="Done","✓ Done",IF(E153="Blocked","Blocked",IF(H153="","No due date",IF(H153&lt;NOW(),"Overdue",IF(H153-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B153="","",IF(E153="Done","Complete",IF(E153="Blocked","Blocked",IF(H153="","No due date",IF(H153&lt;NOW(),"Overdue",IF(H153-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N153" s="51" t="n"/>
@@ -8852,7 +8887,7 @@
         <v/>
       </c>
       <c r="M154" s="58">
-        <f>IF(B154="","",IF(E154="Done","✓ Done",IF(E154="Blocked","Blocked",IF(H154="","No due date",IF(H154&lt;NOW(),"Overdue",IF(H154-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B154="","",IF(E154="Done","Complete",IF(E154="Blocked","Blocked",IF(H154="","No due date",IF(H154&lt;NOW(),"Overdue",IF(H154-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N154" s="51" t="n"/>
@@ -8882,7 +8917,7 @@
         <v/>
       </c>
       <c r="M155" s="58">
-        <f>IF(B155="","",IF(E155="Done","✓ Done",IF(E155="Blocked","Blocked",IF(H155="","No due date",IF(H155&lt;NOW(),"Overdue",IF(H155-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B155="","",IF(E155="Done","Complete",IF(E155="Blocked","Blocked",IF(H155="","No due date",IF(H155&lt;NOW(),"Overdue",IF(H155-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N155" s="51" t="n"/>
@@ -8912,7 +8947,7 @@
         <v/>
       </c>
       <c r="M156" s="58">
-        <f>IF(B156="","",IF(E156="Done","✓ Done",IF(E156="Blocked","Blocked",IF(H156="","No due date",IF(H156&lt;NOW(),"Overdue",IF(H156-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B156="","",IF(E156="Done","Complete",IF(E156="Blocked","Blocked",IF(H156="","No due date",IF(H156&lt;NOW(),"Overdue",IF(H156-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N156" s="51" t="n"/>
@@ -8942,7 +8977,7 @@
         <v/>
       </c>
       <c r="M157" s="58">
-        <f>IF(B157="","",IF(E157="Done","✓ Done",IF(E157="Blocked","Blocked",IF(H157="","No due date",IF(H157&lt;NOW(),"Overdue",IF(H157-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B157="","",IF(E157="Done","Complete",IF(E157="Blocked","Blocked",IF(H157="","No due date",IF(H157&lt;NOW(),"Overdue",IF(H157-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N157" s="51" t="n"/>
@@ -8972,7 +9007,7 @@
         <v/>
       </c>
       <c r="M158" s="58">
-        <f>IF(B158="","",IF(E158="Done","✓ Done",IF(E158="Blocked","Blocked",IF(H158="","No due date",IF(H158&lt;NOW(),"Overdue",IF(H158-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B158="","",IF(E158="Done","Complete",IF(E158="Blocked","Blocked",IF(H158="","No due date",IF(H158&lt;NOW(),"Overdue",IF(H158-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N158" s="51" t="n"/>
@@ -9002,7 +9037,7 @@
         <v/>
       </c>
       <c r="M159" s="58">
-        <f>IF(B159="","",IF(E159="Done","✓ Done",IF(E159="Blocked","Blocked",IF(H159="","No due date",IF(H159&lt;NOW(),"Overdue",IF(H159-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B159="","",IF(E159="Done","Complete",IF(E159="Blocked","Blocked",IF(H159="","No due date",IF(H159&lt;NOW(),"Overdue",IF(H159-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N159" s="51" t="n"/>
@@ -9032,7 +9067,7 @@
         <v/>
       </c>
       <c r="M160" s="58">
-        <f>IF(B160="","",IF(E160="Done","✓ Done",IF(E160="Blocked","Blocked",IF(H160="","No due date",IF(H160&lt;NOW(),"Overdue",IF(H160-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B160="","",IF(E160="Done","Complete",IF(E160="Blocked","Blocked",IF(H160="","No due date",IF(H160&lt;NOW(),"Overdue",IF(H160-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N160" s="51" t="n"/>
@@ -9062,7 +9097,7 @@
         <v/>
       </c>
       <c r="M161" s="58">
-        <f>IF(B161="","",IF(E161="Done","✓ Done",IF(E161="Blocked","Blocked",IF(H161="","No due date",IF(H161&lt;NOW(),"Overdue",IF(H161-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B161="","",IF(E161="Done","Complete",IF(E161="Blocked","Blocked",IF(H161="","No due date",IF(H161&lt;NOW(),"Overdue",IF(H161-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N161" s="51" t="n"/>
@@ -9092,7 +9127,7 @@
         <v/>
       </c>
       <c r="M162" s="58">
-        <f>IF(B162="","",IF(E162="Done","✓ Done",IF(E162="Blocked","Blocked",IF(H162="","No due date",IF(H162&lt;NOW(),"Overdue",IF(H162-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B162="","",IF(E162="Done","Complete",IF(E162="Blocked","Blocked",IF(H162="","No due date",IF(H162&lt;NOW(),"Overdue",IF(H162-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N162" s="51" t="n"/>
@@ -9122,7 +9157,7 @@
         <v/>
       </c>
       <c r="M163" s="58">
-        <f>IF(B163="","",IF(E163="Done","✓ Done",IF(E163="Blocked","Blocked",IF(H163="","No due date",IF(H163&lt;NOW(),"Overdue",IF(H163-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B163="","",IF(E163="Done","Complete",IF(E163="Blocked","Blocked",IF(H163="","No due date",IF(H163&lt;NOW(),"Overdue",IF(H163-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N163" s="51" t="n"/>
@@ -9152,7 +9187,7 @@
         <v/>
       </c>
       <c r="M164" s="58">
-        <f>IF(B164="","",IF(E164="Done","✓ Done",IF(E164="Blocked","Blocked",IF(H164="","No due date",IF(H164&lt;NOW(),"Overdue",IF(H164-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B164="","",IF(E164="Done","Complete",IF(E164="Blocked","Blocked",IF(H164="","No due date",IF(H164&lt;NOW(),"Overdue",IF(H164-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N164" s="51" t="n"/>
@@ -9182,7 +9217,7 @@
         <v/>
       </c>
       <c r="M165" s="58">
-        <f>IF(B165="","",IF(E165="Done","✓ Done",IF(E165="Blocked","Blocked",IF(H165="","No due date",IF(H165&lt;NOW(),"Overdue",IF(H165-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B165="","",IF(E165="Done","Complete",IF(E165="Blocked","Blocked",IF(H165="","No due date",IF(H165&lt;NOW(),"Overdue",IF(H165-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N165" s="51" t="n"/>
@@ -9212,7 +9247,7 @@
         <v/>
       </c>
       <c r="M166" s="58">
-        <f>IF(B166="","",IF(E166="Done","✓ Done",IF(E166="Blocked","Blocked",IF(H166="","No due date",IF(H166&lt;NOW(),"Overdue",IF(H166-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B166="","",IF(E166="Done","Complete",IF(E166="Blocked","Blocked",IF(H166="","No due date",IF(H166&lt;NOW(),"Overdue",IF(H166-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N166" s="51" t="n"/>
@@ -9242,7 +9277,7 @@
         <v/>
       </c>
       <c r="M167" s="58">
-        <f>IF(B167="","",IF(E167="Done","✓ Done",IF(E167="Blocked","Blocked",IF(H167="","No due date",IF(H167&lt;NOW(),"Overdue",IF(H167-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B167="","",IF(E167="Done","Complete",IF(E167="Blocked","Blocked",IF(H167="","No due date",IF(H167&lt;NOW(),"Overdue",IF(H167-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N167" s="51" t="n"/>
@@ -9272,7 +9307,7 @@
         <v/>
       </c>
       <c r="M168" s="58">
-        <f>IF(B168="","",IF(E168="Done","✓ Done",IF(E168="Blocked","Blocked",IF(H168="","No due date",IF(H168&lt;NOW(),"Overdue",IF(H168-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B168="","",IF(E168="Done","Complete",IF(E168="Blocked","Blocked",IF(H168="","No due date",IF(H168&lt;NOW(),"Overdue",IF(H168-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N168" s="51" t="n"/>
@@ -9302,7 +9337,7 @@
         <v/>
       </c>
       <c r="M169" s="58">
-        <f>IF(B169="","",IF(E169="Done","✓ Done",IF(E169="Blocked","Blocked",IF(H169="","No due date",IF(H169&lt;NOW(),"Overdue",IF(H169-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B169="","",IF(E169="Done","Complete",IF(E169="Blocked","Blocked",IF(H169="","No due date",IF(H169&lt;NOW(),"Overdue",IF(H169-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N169" s="51" t="n"/>
@@ -9332,7 +9367,7 @@
         <v/>
       </c>
       <c r="M170" s="58">
-        <f>IF(B170="","",IF(E170="Done","✓ Done",IF(E170="Blocked","Blocked",IF(H170="","No due date",IF(H170&lt;NOW(),"Overdue",IF(H170-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B170="","",IF(E170="Done","Complete",IF(E170="Blocked","Blocked",IF(H170="","No due date",IF(H170&lt;NOW(),"Overdue",IF(H170-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N170" s="51" t="n"/>
@@ -9362,7 +9397,7 @@
         <v/>
       </c>
       <c r="M171" s="58">
-        <f>IF(B171="","",IF(E171="Done","✓ Done",IF(E171="Blocked","Blocked",IF(H171="","No due date",IF(H171&lt;NOW(),"Overdue",IF(H171-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B171="","",IF(E171="Done","Complete",IF(E171="Blocked","Blocked",IF(H171="","No due date",IF(H171&lt;NOW(),"Overdue",IF(H171-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N171" s="51" t="n"/>
@@ -9392,7 +9427,7 @@
         <v/>
       </c>
       <c r="M172" s="58">
-        <f>IF(B172="","",IF(E172="Done","✓ Done",IF(E172="Blocked","Blocked",IF(H172="","No due date",IF(H172&lt;NOW(),"Overdue",IF(H172-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B172="","",IF(E172="Done","Complete",IF(E172="Blocked","Blocked",IF(H172="","No due date",IF(H172&lt;NOW(),"Overdue",IF(H172-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N172" s="51" t="n"/>
@@ -9422,7 +9457,7 @@
         <v/>
       </c>
       <c r="M173" s="58">
-        <f>IF(B173="","",IF(E173="Done","✓ Done",IF(E173="Blocked","Blocked",IF(H173="","No due date",IF(H173&lt;NOW(),"Overdue",IF(H173-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B173="","",IF(E173="Done","Complete",IF(E173="Blocked","Blocked",IF(H173="","No due date",IF(H173&lt;NOW(),"Overdue",IF(H173-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N173" s="51" t="n"/>
@@ -9452,7 +9487,7 @@
         <v/>
       </c>
       <c r="M174" s="58">
-        <f>IF(B174="","",IF(E174="Done","✓ Done",IF(E174="Blocked","Blocked",IF(H174="","No due date",IF(H174&lt;NOW(),"Overdue",IF(H174-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B174="","",IF(E174="Done","Complete",IF(E174="Blocked","Blocked",IF(H174="","No due date",IF(H174&lt;NOW(),"Overdue",IF(H174-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N174" s="51" t="n"/>
@@ -9482,7 +9517,7 @@
         <v/>
       </c>
       <c r="M175" s="58">
-        <f>IF(B175="","",IF(E175="Done","✓ Done",IF(E175="Blocked","Blocked",IF(H175="","No due date",IF(H175&lt;NOW(),"Overdue",IF(H175-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B175="","",IF(E175="Done","Complete",IF(E175="Blocked","Blocked",IF(H175="","No due date",IF(H175&lt;NOW(),"Overdue",IF(H175-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N175" s="51" t="n"/>
@@ -9512,7 +9547,7 @@
         <v/>
       </c>
       <c r="M176" s="58">
-        <f>IF(B176="","",IF(E176="Done","✓ Done",IF(E176="Blocked","Blocked",IF(H176="","No due date",IF(H176&lt;NOW(),"Overdue",IF(H176-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B176="","",IF(E176="Done","Complete",IF(E176="Blocked","Blocked",IF(H176="","No due date",IF(H176&lt;NOW(),"Overdue",IF(H176-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N176" s="51" t="n"/>
@@ -9542,7 +9577,7 @@
         <v/>
       </c>
       <c r="M177" s="58">
-        <f>IF(B177="","",IF(E177="Done","✓ Done",IF(E177="Blocked","Blocked",IF(H177="","No due date",IF(H177&lt;NOW(),"Overdue",IF(H177-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B177="","",IF(E177="Done","Complete",IF(E177="Blocked","Blocked",IF(H177="","No due date",IF(H177&lt;NOW(),"Overdue",IF(H177-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N177" s="51" t="n"/>
@@ -9572,7 +9607,7 @@
         <v/>
       </c>
       <c r="M178" s="58">
-        <f>IF(B178="","",IF(E178="Done","✓ Done",IF(E178="Blocked","Blocked",IF(H178="","No due date",IF(H178&lt;NOW(),"Overdue",IF(H178-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B178="","",IF(E178="Done","Complete",IF(E178="Blocked","Blocked",IF(H178="","No due date",IF(H178&lt;NOW(),"Overdue",IF(H178-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N178" s="51" t="n"/>
@@ -9602,7 +9637,7 @@
         <v/>
       </c>
       <c r="M179" s="58">
-        <f>IF(B179="","",IF(E179="Done","✓ Done",IF(E179="Blocked","Blocked",IF(H179="","No due date",IF(H179&lt;NOW(),"Overdue",IF(H179-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B179="","",IF(E179="Done","Complete",IF(E179="Blocked","Blocked",IF(H179="","No due date",IF(H179&lt;NOW(),"Overdue",IF(H179-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N179" s="51" t="n"/>
@@ -9632,7 +9667,7 @@
         <v/>
       </c>
       <c r="M180" s="58">
-        <f>IF(B180="","",IF(E180="Done","✓ Done",IF(E180="Blocked","Blocked",IF(H180="","No due date",IF(H180&lt;NOW(),"Overdue",IF(H180-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B180="","",IF(E180="Done","Complete",IF(E180="Blocked","Blocked",IF(H180="","No due date",IF(H180&lt;NOW(),"Overdue",IF(H180-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N180" s="51" t="n"/>
@@ -9662,7 +9697,7 @@
         <v/>
       </c>
       <c r="M181" s="58">
-        <f>IF(B181="","",IF(E181="Done","✓ Done",IF(E181="Blocked","Blocked",IF(H181="","No due date",IF(H181&lt;NOW(),"Overdue",IF(H181-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B181="","",IF(E181="Done","Complete",IF(E181="Blocked","Blocked",IF(H181="","No due date",IF(H181&lt;NOW(),"Overdue",IF(H181-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N181" s="51" t="n"/>
@@ -9692,7 +9727,7 @@
         <v/>
       </c>
       <c r="M182" s="58">
-        <f>IF(B182="","",IF(E182="Done","✓ Done",IF(E182="Blocked","Blocked",IF(H182="","No due date",IF(H182&lt;NOW(),"Overdue",IF(H182-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B182="","",IF(E182="Done","Complete",IF(E182="Blocked","Blocked",IF(H182="","No due date",IF(H182&lt;NOW(),"Overdue",IF(H182-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N182" s="51" t="n"/>
@@ -9722,7 +9757,7 @@
         <v/>
       </c>
       <c r="M183" s="58">
-        <f>IF(B183="","",IF(E183="Done","✓ Done",IF(E183="Blocked","Blocked",IF(H183="","No due date",IF(H183&lt;NOW(),"Overdue",IF(H183-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B183="","",IF(E183="Done","Complete",IF(E183="Blocked","Blocked",IF(H183="","No due date",IF(H183&lt;NOW(),"Overdue",IF(H183-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N183" s="51" t="n"/>
@@ -9752,7 +9787,7 @@
         <v/>
       </c>
       <c r="M184" s="58">
-        <f>IF(B184="","",IF(E184="Done","✓ Done",IF(E184="Blocked","Blocked",IF(H184="","No due date",IF(H184&lt;NOW(),"Overdue",IF(H184-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B184="","",IF(E184="Done","Complete",IF(E184="Blocked","Blocked",IF(H184="","No due date",IF(H184&lt;NOW(),"Overdue",IF(H184-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N184" s="51" t="n"/>
@@ -9782,7 +9817,7 @@
         <v/>
       </c>
       <c r="M185" s="58">
-        <f>IF(B185="","",IF(E185="Done","✓ Done",IF(E185="Blocked","Blocked",IF(H185="","No due date",IF(H185&lt;NOW(),"Overdue",IF(H185-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B185="","",IF(E185="Done","Complete",IF(E185="Blocked","Blocked",IF(H185="","No due date",IF(H185&lt;NOW(),"Overdue",IF(H185-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N185" s="51" t="n"/>
@@ -9812,7 +9847,7 @@
         <v/>
       </c>
       <c r="M186" s="58">
-        <f>IF(B186="","",IF(E186="Done","✓ Done",IF(E186="Blocked","Blocked",IF(H186="","No due date",IF(H186&lt;NOW(),"Overdue",IF(H186-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B186="","",IF(E186="Done","Complete",IF(E186="Blocked","Blocked",IF(H186="","No due date",IF(H186&lt;NOW(),"Overdue",IF(H186-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N186" s="51" t="n"/>
@@ -9842,7 +9877,7 @@
         <v/>
       </c>
       <c r="M187" s="58">
-        <f>IF(B187="","",IF(E187="Done","✓ Done",IF(E187="Blocked","Blocked",IF(H187="","No due date",IF(H187&lt;NOW(),"Overdue",IF(H187-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B187="","",IF(E187="Done","Complete",IF(E187="Blocked","Blocked",IF(H187="","No due date",IF(H187&lt;NOW(),"Overdue",IF(H187-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N187" s="51" t="n"/>
@@ -9872,7 +9907,7 @@
         <v/>
       </c>
       <c r="M188" s="58">
-        <f>IF(B188="","",IF(E188="Done","✓ Done",IF(E188="Blocked","Blocked",IF(H188="","No due date",IF(H188&lt;NOW(),"Overdue",IF(H188-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B188="","",IF(E188="Done","Complete",IF(E188="Blocked","Blocked",IF(H188="","No due date",IF(H188&lt;NOW(),"Overdue",IF(H188-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N188" s="51" t="n"/>
@@ -9902,7 +9937,7 @@
         <v/>
       </c>
       <c r="M189" s="58">
-        <f>IF(B189="","",IF(E189="Done","✓ Done",IF(E189="Blocked","Blocked",IF(H189="","No due date",IF(H189&lt;NOW(),"Overdue",IF(H189-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B189="","",IF(E189="Done","Complete",IF(E189="Blocked","Blocked",IF(H189="","No due date",IF(H189&lt;NOW(),"Overdue",IF(H189-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N189" s="51" t="n"/>
@@ -9932,7 +9967,7 @@
         <v/>
       </c>
       <c r="M190" s="58">
-        <f>IF(B190="","",IF(E190="Done","✓ Done",IF(E190="Blocked","Blocked",IF(H190="","No due date",IF(H190&lt;NOW(),"Overdue",IF(H190-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B190="","",IF(E190="Done","Complete",IF(E190="Blocked","Blocked",IF(H190="","No due date",IF(H190&lt;NOW(),"Overdue",IF(H190-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N190" s="51" t="n"/>
@@ -9962,7 +9997,7 @@
         <v/>
       </c>
       <c r="M191" s="58">
-        <f>IF(B191="","",IF(E191="Done","✓ Done",IF(E191="Blocked","Blocked",IF(H191="","No due date",IF(H191&lt;NOW(),"Overdue",IF(H191-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B191="","",IF(E191="Done","Complete",IF(E191="Blocked","Blocked",IF(H191="","No due date",IF(H191&lt;NOW(),"Overdue",IF(H191-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N191" s="51" t="n"/>
@@ -9992,7 +10027,7 @@
         <v/>
       </c>
       <c r="M192" s="58">
-        <f>IF(B192="","",IF(E192="Done","✓ Done",IF(E192="Blocked","Blocked",IF(H192="","No due date",IF(H192&lt;NOW(),"Overdue",IF(H192-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B192="","",IF(E192="Done","Complete",IF(E192="Blocked","Blocked",IF(H192="","No due date",IF(H192&lt;NOW(),"Overdue",IF(H192-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N192" s="51" t="n"/>
@@ -10022,7 +10057,7 @@
         <v/>
       </c>
       <c r="M193" s="58">
-        <f>IF(B193="","",IF(E193="Done","✓ Done",IF(E193="Blocked","Blocked",IF(H193="","No due date",IF(H193&lt;NOW(),"Overdue",IF(H193-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B193="","",IF(E193="Done","Complete",IF(E193="Blocked","Blocked",IF(H193="","No due date",IF(H193&lt;NOW(),"Overdue",IF(H193-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N193" s="51" t="n"/>
@@ -10052,7 +10087,7 @@
         <v/>
       </c>
       <c r="M194" s="58">
-        <f>IF(B194="","",IF(E194="Done","✓ Done",IF(E194="Blocked","Blocked",IF(H194="","No due date",IF(H194&lt;NOW(),"Overdue",IF(H194-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B194="","",IF(E194="Done","Complete",IF(E194="Blocked","Blocked",IF(H194="","No due date",IF(H194&lt;NOW(),"Overdue",IF(H194-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N194" s="51" t="n"/>
@@ -10082,7 +10117,7 @@
         <v/>
       </c>
       <c r="M195" s="58">
-        <f>IF(B195="","",IF(E195="Done","✓ Done",IF(E195="Blocked","Blocked",IF(H195="","No due date",IF(H195&lt;NOW(),"Overdue",IF(H195-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B195="","",IF(E195="Done","Complete",IF(E195="Blocked","Blocked",IF(H195="","No due date",IF(H195&lt;NOW(),"Overdue",IF(H195-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N195" s="51" t="n"/>
@@ -10112,7 +10147,7 @@
         <v/>
       </c>
       <c r="M196" s="58">
-        <f>IF(B196="","",IF(E196="Done","✓ Done",IF(E196="Blocked","Blocked",IF(H196="","No due date",IF(H196&lt;NOW(),"Overdue",IF(H196-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B196="","",IF(E196="Done","Complete",IF(E196="Blocked","Blocked",IF(H196="","No due date",IF(H196&lt;NOW(),"Overdue",IF(H196-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N196" s="51" t="n"/>
@@ -10142,7 +10177,7 @@
         <v/>
       </c>
       <c r="M197" s="58">
-        <f>IF(B197="","",IF(E197="Done","✓ Done",IF(E197="Blocked","Blocked",IF(H197="","No due date",IF(H197&lt;NOW(),"Overdue",IF(H197-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B197="","",IF(E197="Done","Complete",IF(E197="Blocked","Blocked",IF(H197="","No due date",IF(H197&lt;NOW(),"Overdue",IF(H197-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N197" s="51" t="n"/>
@@ -10172,7 +10207,7 @@
         <v/>
       </c>
       <c r="M198" s="58">
-        <f>IF(B198="","",IF(E198="Done","✓ Done",IF(E198="Blocked","Blocked",IF(H198="","No due date",IF(H198&lt;NOW(),"Overdue",IF(H198-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B198="","",IF(E198="Done","Complete",IF(E198="Blocked","Blocked",IF(H198="","No due date",IF(H198&lt;NOW(),"Overdue",IF(H198-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N198" s="51" t="n"/>
@@ -10202,7 +10237,7 @@
         <v/>
       </c>
       <c r="M199" s="58">
-        <f>IF(B199="","",IF(E199="Done","✓ Done",IF(E199="Blocked","Blocked",IF(H199="","No due date",IF(H199&lt;NOW(),"Overdue",IF(H199-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B199="","",IF(E199="Done","Complete",IF(E199="Blocked","Blocked",IF(H199="","No due date",IF(H199&lt;NOW(),"Overdue",IF(H199-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N199" s="51" t="n"/>
@@ -10232,7 +10267,7 @@
         <v/>
       </c>
       <c r="M200" s="58">
-        <f>IF(B200="","",IF(E200="Done","✓ Done",IF(E200="Blocked","Blocked",IF(H200="","No due date",IF(H200&lt;NOW(),"Overdue",IF(H200-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B200="","",IF(E200="Done","Complete",IF(E200="Blocked","Blocked",IF(H200="","No due date",IF(H200&lt;NOW(),"Overdue",IF(H200-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N200" s="51" t="n"/>
@@ -10262,7 +10297,7 @@
         <v/>
       </c>
       <c r="M201" s="58">
-        <f>IF(B201="","",IF(E201="Done","✓ Done",IF(E201="Blocked","Blocked",IF(H201="","No due date",IF(H201&lt;NOW(),"Overdue",IF(H201-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B201="","",IF(E201="Done","Complete",IF(E201="Blocked","Blocked",IF(H201="","No due date",IF(H201&lt;NOW(),"Overdue",IF(H201-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N201" s="51" t="n"/>
@@ -10292,7 +10327,7 @@
         <v/>
       </c>
       <c r="M202" s="58">
-        <f>IF(B202="","",IF(E202="Done","✓ Done",IF(E202="Blocked","Blocked",IF(H202="","No due date",IF(H202&lt;NOW(),"Overdue",IF(H202-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B202="","",IF(E202="Done","Complete",IF(E202="Blocked","Blocked",IF(H202="","No due date",IF(H202&lt;NOW(),"Overdue",IF(H202-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N202" s="51" t="n"/>
@@ -10322,7 +10357,7 @@
         <v/>
       </c>
       <c r="M203" s="58">
-        <f>IF(B203="","",IF(E203="Done","✓ Done",IF(E203="Blocked","Blocked",IF(H203="","No due date",IF(H203&lt;NOW(),"Overdue",IF(H203-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B203="","",IF(E203="Done","Complete",IF(E203="Blocked","Blocked",IF(H203="","No due date",IF(H203&lt;NOW(),"Overdue",IF(H203-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N203" s="51" t="n"/>
@@ -10352,7 +10387,7 @@
         <v/>
       </c>
       <c r="M204" s="58">
-        <f>IF(B204="","",IF(E204="Done","✓ Done",IF(E204="Blocked","Blocked",IF(H204="","No due date",IF(H204&lt;NOW(),"Overdue",IF(H204-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B204="","",IF(E204="Done","Complete",IF(E204="Blocked","Blocked",IF(H204="","No due date",IF(H204&lt;NOW(),"Overdue",IF(H204-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N204" s="51" t="n"/>
@@ -10382,7 +10417,7 @@
         <v/>
       </c>
       <c r="M205" s="58">
-        <f>IF(B205="","",IF(E205="Done","✓ Done",IF(E205="Blocked","Blocked",IF(H205="","No due date",IF(H205&lt;NOW(),"Overdue",IF(H205-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B205="","",IF(E205="Done","Complete",IF(E205="Blocked","Blocked",IF(H205="","No due date",IF(H205&lt;NOW(),"Overdue",IF(H205-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N205" s="51" t="n"/>
@@ -10412,7 +10447,7 @@
         <v/>
       </c>
       <c r="M206" s="58">
-        <f>IF(B206="","",IF(E206="Done","✓ Done",IF(E206="Blocked","Blocked",IF(H206="","No due date",IF(H206&lt;NOW(),"Overdue",IF(H206-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B206="","",IF(E206="Done","Complete",IF(E206="Blocked","Blocked",IF(H206="","No due date",IF(H206&lt;NOW(),"Overdue",IF(H206-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N206" s="51" t="n"/>
@@ -10442,7 +10477,7 @@
         <v/>
       </c>
       <c r="M207" s="58">
-        <f>IF(B207="","",IF(E207="Done","✓ Done",IF(E207="Blocked","Blocked",IF(H207="","No due date",IF(H207&lt;NOW(),"Overdue",IF(H207-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B207="","",IF(E207="Done","Complete",IF(E207="Blocked","Blocked",IF(H207="","No due date",IF(H207&lt;NOW(),"Overdue",IF(H207-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N207" s="51" t="n"/>
@@ -10472,7 +10507,7 @@
         <v/>
       </c>
       <c r="M208" s="58">
-        <f>IF(B208="","",IF(E208="Done","✓ Done",IF(E208="Blocked","Blocked",IF(H208="","No due date",IF(H208&lt;NOW(),"Overdue",IF(H208-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B208="","",IF(E208="Done","Complete",IF(E208="Blocked","Blocked",IF(H208="","No due date",IF(H208&lt;NOW(),"Overdue",IF(H208-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N208" s="51" t="n"/>
@@ -10502,7 +10537,7 @@
         <v/>
       </c>
       <c r="M209" s="58">
-        <f>IF(B209="","",IF(E209="Done","✓ Done",IF(E209="Blocked","Blocked",IF(H209="","No due date",IF(H209&lt;NOW(),"Overdue",IF(H209-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B209="","",IF(E209="Done","Complete",IF(E209="Blocked","Blocked",IF(H209="","No due date",IF(H209&lt;NOW(),"Overdue",IF(H209-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N209" s="51" t="n"/>
@@ -10532,7 +10567,7 @@
         <v/>
       </c>
       <c r="M210" s="58">
-        <f>IF(B210="","",IF(E210="Done","✓ Done",IF(E210="Blocked","Blocked",IF(H210="","No due date",IF(H210&lt;NOW(),"Overdue",IF(H210-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B210="","",IF(E210="Done","Complete",IF(E210="Blocked","Blocked",IF(H210="","No due date",IF(H210&lt;NOW(),"Overdue",IF(H210-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N210" s="51" t="n"/>
@@ -10562,7 +10597,7 @@
         <v/>
       </c>
       <c r="M211" s="58">
-        <f>IF(B211="","",IF(E211="Done","✓ Done",IF(E211="Blocked","Blocked",IF(H211="","No due date",IF(H211&lt;NOW(),"Overdue",IF(H211-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B211="","",IF(E211="Done","Complete",IF(E211="Blocked","Blocked",IF(H211="","No due date",IF(H211&lt;NOW(),"Overdue",IF(H211-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N211" s="51" t="n"/>
@@ -10592,7 +10627,7 @@
         <v/>
       </c>
       <c r="M212" s="58">
-        <f>IF(B212="","",IF(E212="Done","✓ Done",IF(E212="Blocked","Blocked",IF(H212="","No due date",IF(H212&lt;NOW(),"Overdue",IF(H212-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B212="","",IF(E212="Done","Complete",IF(E212="Blocked","Blocked",IF(H212="","No due date",IF(H212&lt;NOW(),"Overdue",IF(H212-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N212" s="51" t="n"/>
@@ -10622,7 +10657,7 @@
         <v/>
       </c>
       <c r="M213" s="58">
-        <f>IF(B213="","",IF(E213="Done","✓ Done",IF(E213="Blocked","Blocked",IF(H213="","No due date",IF(H213&lt;NOW(),"Overdue",IF(H213-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B213="","",IF(E213="Done","Complete",IF(E213="Blocked","Blocked",IF(H213="","No due date",IF(H213&lt;NOW(),"Overdue",IF(H213-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N213" s="51" t="n"/>
@@ -10652,7 +10687,7 @@
         <v/>
       </c>
       <c r="M214" s="58">
-        <f>IF(B214="","",IF(E214="Done","✓ Done",IF(E214="Blocked","Blocked",IF(H214="","No due date",IF(H214&lt;NOW(),"Overdue",IF(H214-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B214="","",IF(E214="Done","Complete",IF(E214="Blocked","Blocked",IF(H214="","No due date",IF(H214&lt;NOW(),"Overdue",IF(H214-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N214" s="51" t="n"/>
@@ -10682,7 +10717,7 @@
         <v/>
       </c>
       <c r="M215" s="58">
-        <f>IF(B215="","",IF(E215="Done","✓ Done",IF(E215="Blocked","Blocked",IF(H215="","No due date",IF(H215&lt;NOW(),"Overdue",IF(H215-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B215="","",IF(E215="Done","Complete",IF(E215="Blocked","Blocked",IF(H215="","No due date",IF(H215&lt;NOW(),"Overdue",IF(H215-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N215" s="51" t="n"/>
@@ -10712,7 +10747,7 @@
         <v/>
       </c>
       <c r="M216" s="58">
-        <f>IF(B216="","",IF(E216="Done","✓ Done",IF(E216="Blocked","Blocked",IF(H216="","No due date",IF(H216&lt;NOW(),"Overdue",IF(H216-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B216="","",IF(E216="Done","Complete",IF(E216="Blocked","Blocked",IF(H216="","No due date",IF(H216&lt;NOW(),"Overdue",IF(H216-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N216" s="51" t="n"/>
@@ -10742,7 +10777,7 @@
         <v/>
       </c>
       <c r="M217" s="58">
-        <f>IF(B217="","",IF(E217="Done","✓ Done",IF(E217="Blocked","Blocked",IF(H217="","No due date",IF(H217&lt;NOW(),"Overdue",IF(H217-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B217="","",IF(E217="Done","Complete",IF(E217="Blocked","Blocked",IF(H217="","No due date",IF(H217&lt;NOW(),"Overdue",IF(H217-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N217" s="51" t="n"/>
@@ -10772,7 +10807,7 @@
         <v/>
       </c>
       <c r="M218" s="58">
-        <f>IF(B218="","",IF(E218="Done","✓ Done",IF(E218="Blocked","Blocked",IF(H218="","No due date",IF(H218&lt;NOW(),"Overdue",IF(H218-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B218="","",IF(E218="Done","Complete",IF(E218="Blocked","Blocked",IF(H218="","No due date",IF(H218&lt;NOW(),"Overdue",IF(H218-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N218" s="51" t="n"/>
@@ -10802,7 +10837,7 @@
         <v/>
       </c>
       <c r="M219" s="58">
-        <f>IF(B219="","",IF(E219="Done","✓ Done",IF(E219="Blocked","Blocked",IF(H219="","No due date",IF(H219&lt;NOW(),"Overdue",IF(H219-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B219="","",IF(E219="Done","Complete",IF(E219="Blocked","Blocked",IF(H219="","No due date",IF(H219&lt;NOW(),"Overdue",IF(H219-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N219" s="51" t="n"/>
@@ -10832,7 +10867,7 @@
         <v/>
       </c>
       <c r="M220" s="58">
-        <f>IF(B220="","",IF(E220="Done","✓ Done",IF(E220="Blocked","Blocked",IF(H220="","No due date",IF(H220&lt;NOW(),"Overdue",IF(H220-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B220="","",IF(E220="Done","Complete",IF(E220="Blocked","Blocked",IF(H220="","No due date",IF(H220&lt;NOW(),"Overdue",IF(H220-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N220" s="51" t="n"/>
@@ -10862,7 +10897,7 @@
         <v/>
       </c>
       <c r="M221" s="58">
-        <f>IF(B221="","",IF(E221="Done","✓ Done",IF(E221="Blocked","Blocked",IF(H221="","No due date",IF(H221&lt;NOW(),"Overdue",IF(H221-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B221="","",IF(E221="Done","Complete",IF(E221="Blocked","Blocked",IF(H221="","No due date",IF(H221&lt;NOW(),"Overdue",IF(H221-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N221" s="51" t="n"/>
@@ -10892,7 +10927,7 @@
         <v/>
       </c>
       <c r="M222" s="58">
-        <f>IF(B222="","",IF(E222="Done","✓ Done",IF(E222="Blocked","Blocked",IF(H222="","No due date",IF(H222&lt;NOW(),"Overdue",IF(H222-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B222="","",IF(E222="Done","Complete",IF(E222="Blocked","Blocked",IF(H222="","No due date",IF(H222&lt;NOW(),"Overdue",IF(H222-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N222" s="51" t="n"/>
@@ -10922,7 +10957,7 @@
         <v/>
       </c>
       <c r="M223" s="58">
-        <f>IF(B223="","",IF(E223="Done","✓ Done",IF(E223="Blocked","Blocked",IF(H223="","No due date",IF(H223&lt;NOW(),"Overdue",IF(H223-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B223="","",IF(E223="Done","Complete",IF(E223="Blocked","Blocked",IF(H223="","No due date",IF(H223&lt;NOW(),"Overdue",IF(H223-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N223" s="51" t="n"/>
@@ -10952,7 +10987,7 @@
         <v/>
       </c>
       <c r="M224" s="58">
-        <f>IF(B224="","",IF(E224="Done","✓ Done",IF(E224="Blocked","Blocked",IF(H224="","No due date",IF(H224&lt;NOW(),"Overdue",IF(H224-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B224="","",IF(E224="Done","Complete",IF(E224="Blocked","Blocked",IF(H224="","No due date",IF(H224&lt;NOW(),"Overdue",IF(H224-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N224" s="51" t="n"/>
@@ -10982,7 +11017,7 @@
         <v/>
       </c>
       <c r="M225" s="58">
-        <f>IF(B225="","",IF(E225="Done","✓ Done",IF(E225="Blocked","Blocked",IF(H225="","No due date",IF(H225&lt;NOW(),"Overdue",IF(H225-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B225="","",IF(E225="Done","Complete",IF(E225="Blocked","Blocked",IF(H225="","No due date",IF(H225&lt;NOW(),"Overdue",IF(H225-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N225" s="51" t="n"/>
@@ -11012,7 +11047,7 @@
         <v/>
       </c>
       <c r="M226" s="58">
-        <f>IF(B226="","",IF(E226="Done","✓ Done",IF(E226="Blocked","Blocked",IF(H226="","No due date",IF(H226&lt;NOW(),"Overdue",IF(H226-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B226="","",IF(E226="Done","Complete",IF(E226="Blocked","Blocked",IF(H226="","No due date",IF(H226&lt;NOW(),"Overdue",IF(H226-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N226" s="51" t="n"/>
@@ -11042,7 +11077,7 @@
         <v/>
       </c>
       <c r="M227" s="58">
-        <f>IF(B227="","",IF(E227="Done","✓ Done",IF(E227="Blocked","Blocked",IF(H227="","No due date",IF(H227&lt;NOW(),"Overdue",IF(H227-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B227="","",IF(E227="Done","Complete",IF(E227="Blocked","Blocked",IF(H227="","No due date",IF(H227&lt;NOW(),"Overdue",IF(H227-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N227" s="51" t="n"/>
@@ -11072,7 +11107,7 @@
         <v/>
       </c>
       <c r="M228" s="58">
-        <f>IF(B228="","",IF(E228="Done","✓ Done",IF(E228="Blocked","Blocked",IF(H228="","No due date",IF(H228&lt;NOW(),"Overdue",IF(H228-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B228="","",IF(E228="Done","Complete",IF(E228="Blocked","Blocked",IF(H228="","No due date",IF(H228&lt;NOW(),"Overdue",IF(H228-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N228" s="51" t="n"/>
@@ -11102,7 +11137,7 @@
         <v/>
       </c>
       <c r="M229" s="58">
-        <f>IF(B229="","",IF(E229="Done","✓ Done",IF(E229="Blocked","Blocked",IF(H229="","No due date",IF(H229&lt;NOW(),"Overdue",IF(H229-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B229="","",IF(E229="Done","Complete",IF(E229="Blocked","Blocked",IF(H229="","No due date",IF(H229&lt;NOW(),"Overdue",IF(H229-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N229" s="51" t="n"/>
@@ -11132,7 +11167,7 @@
         <v/>
       </c>
       <c r="M230" s="58">
-        <f>IF(B230="","",IF(E230="Done","✓ Done",IF(E230="Blocked","Blocked",IF(H230="","No due date",IF(H230&lt;NOW(),"Overdue",IF(H230-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B230="","",IF(E230="Done","Complete",IF(E230="Blocked","Blocked",IF(H230="","No due date",IF(H230&lt;NOW(),"Overdue",IF(H230-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N230" s="51" t="n"/>
@@ -11162,7 +11197,7 @@
         <v/>
       </c>
       <c r="M231" s="58">
-        <f>IF(B231="","",IF(E231="Done","✓ Done",IF(E231="Blocked","Blocked",IF(H231="","No due date",IF(H231&lt;NOW(),"Overdue",IF(H231-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B231="","",IF(E231="Done","Complete",IF(E231="Blocked","Blocked",IF(H231="","No due date",IF(H231&lt;NOW(),"Overdue",IF(H231-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N231" s="51" t="n"/>
@@ -11192,7 +11227,7 @@
         <v/>
       </c>
       <c r="M232" s="58">
-        <f>IF(B232="","",IF(E232="Done","✓ Done",IF(E232="Blocked","Blocked",IF(H232="","No due date",IF(H232&lt;NOW(),"Overdue",IF(H232-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B232="","",IF(E232="Done","Complete",IF(E232="Blocked","Blocked",IF(H232="","No due date",IF(H232&lt;NOW(),"Overdue",IF(H232-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N232" s="51" t="n"/>
@@ -11222,7 +11257,7 @@
         <v/>
       </c>
       <c r="M233" s="58">
-        <f>IF(B233="","",IF(E233="Done","✓ Done",IF(E233="Blocked","Blocked",IF(H233="","No due date",IF(H233&lt;NOW(),"Overdue",IF(H233-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B233="","",IF(E233="Done","Complete",IF(E233="Blocked","Blocked",IF(H233="","No due date",IF(H233&lt;NOW(),"Overdue",IF(H233-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N233" s="51" t="n"/>
@@ -11252,7 +11287,7 @@
         <v/>
       </c>
       <c r="M234" s="58">
-        <f>IF(B234="","",IF(E234="Done","✓ Done",IF(E234="Blocked","Blocked",IF(H234="","No due date",IF(H234&lt;NOW(),"Overdue",IF(H234-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B234="","",IF(E234="Done","Complete",IF(E234="Blocked","Blocked",IF(H234="","No due date",IF(H234&lt;NOW(),"Overdue",IF(H234-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N234" s="51" t="n"/>
@@ -11282,7 +11317,7 @@
         <v/>
       </c>
       <c r="M235" s="58">
-        <f>IF(B235="","",IF(E235="Done","✓ Done",IF(E235="Blocked","Blocked",IF(H235="","No due date",IF(H235&lt;NOW(),"Overdue",IF(H235-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B235="","",IF(E235="Done","Complete",IF(E235="Blocked","Blocked",IF(H235="","No due date",IF(H235&lt;NOW(),"Overdue",IF(H235-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N235" s="51" t="n"/>
@@ -11312,7 +11347,7 @@
         <v/>
       </c>
       <c r="M236" s="58">
-        <f>IF(B236="","",IF(E236="Done","✓ Done",IF(E236="Blocked","Blocked",IF(H236="","No due date",IF(H236&lt;NOW(),"Overdue",IF(H236-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B236="","",IF(E236="Done","Complete",IF(E236="Blocked","Blocked",IF(H236="","No due date",IF(H236&lt;NOW(),"Overdue",IF(H236-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N236" s="51" t="n"/>
@@ -11342,7 +11377,7 @@
         <v/>
       </c>
       <c r="M237" s="58">
-        <f>IF(B237="","",IF(E237="Done","✓ Done",IF(E237="Blocked","Blocked",IF(H237="","No due date",IF(H237&lt;NOW(),"Overdue",IF(H237-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B237="","",IF(E237="Done","Complete",IF(E237="Blocked","Blocked",IF(H237="","No due date",IF(H237&lt;NOW(),"Overdue",IF(H237-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N237" s="51" t="n"/>
@@ -11372,7 +11407,7 @@
         <v/>
       </c>
       <c r="M238" s="58">
-        <f>IF(B238="","",IF(E238="Done","✓ Done",IF(E238="Blocked","Blocked",IF(H238="","No due date",IF(H238&lt;NOW(),"Overdue",IF(H238-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B238="","",IF(E238="Done","Complete",IF(E238="Blocked","Blocked",IF(H238="","No due date",IF(H238&lt;NOW(),"Overdue",IF(H238-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N238" s="51" t="n"/>
@@ -11402,7 +11437,7 @@
         <v/>
       </c>
       <c r="M239" s="58">
-        <f>IF(B239="","",IF(E239="Done","✓ Done",IF(E239="Blocked","Blocked",IF(H239="","No due date",IF(H239&lt;NOW(),"Overdue",IF(H239-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B239="","",IF(E239="Done","Complete",IF(E239="Blocked","Blocked",IF(H239="","No due date",IF(H239&lt;NOW(),"Overdue",IF(H239-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N239" s="51" t="n"/>
@@ -11432,7 +11467,7 @@
         <v/>
       </c>
       <c r="M240" s="58">
-        <f>IF(B240="","",IF(E240="Done","✓ Done",IF(E240="Blocked","Blocked",IF(H240="","No due date",IF(H240&lt;NOW(),"Overdue",IF(H240-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B240="","",IF(E240="Done","Complete",IF(E240="Blocked","Blocked",IF(H240="","No due date",IF(H240&lt;NOW(),"Overdue",IF(H240-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N240" s="51" t="n"/>
@@ -11462,7 +11497,7 @@
         <v/>
       </c>
       <c r="M241" s="58">
-        <f>IF(B241="","",IF(E241="Done","✓ Done",IF(E241="Blocked","Blocked",IF(H241="","No due date",IF(H241&lt;NOW(),"Overdue",IF(H241-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B241="","",IF(E241="Done","Complete",IF(E241="Blocked","Blocked",IF(H241="","No due date",IF(H241&lt;NOW(),"Overdue",IF(H241-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N241" s="51" t="n"/>
@@ -11492,7 +11527,7 @@
         <v/>
       </c>
       <c r="M242" s="58">
-        <f>IF(B242="","",IF(E242="Done","✓ Done",IF(E242="Blocked","Blocked",IF(H242="","No due date",IF(H242&lt;NOW(),"Overdue",IF(H242-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B242="","",IF(E242="Done","Complete",IF(E242="Blocked","Blocked",IF(H242="","No due date",IF(H242&lt;NOW(),"Overdue",IF(H242-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N242" s="51" t="n"/>
@@ -11522,7 +11557,7 @@
         <v/>
       </c>
       <c r="M243" s="58">
-        <f>IF(B243="","",IF(E243="Done","✓ Done",IF(E243="Blocked","Blocked",IF(H243="","No due date",IF(H243&lt;NOW(),"Overdue",IF(H243-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B243="","",IF(E243="Done","Complete",IF(E243="Blocked","Blocked",IF(H243="","No due date",IF(H243&lt;NOW(),"Overdue",IF(H243-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N243" s="51" t="n"/>
@@ -11552,7 +11587,7 @@
         <v/>
       </c>
       <c r="M244" s="58">
-        <f>IF(B244="","",IF(E244="Done","✓ Done",IF(E244="Blocked","Blocked",IF(H244="","No due date",IF(H244&lt;NOW(),"Overdue",IF(H244-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B244="","",IF(E244="Done","Complete",IF(E244="Blocked","Blocked",IF(H244="","No due date",IF(H244&lt;NOW(),"Overdue",IF(H244-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N244" s="51" t="n"/>
@@ -11582,7 +11617,7 @@
         <v/>
       </c>
       <c r="M245" s="58">
-        <f>IF(B245="","",IF(E245="Done","✓ Done",IF(E245="Blocked","Blocked",IF(H245="","No due date",IF(H245&lt;NOW(),"Overdue",IF(H245-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B245="","",IF(E245="Done","Complete",IF(E245="Blocked","Blocked",IF(H245="","No due date",IF(H245&lt;NOW(),"Overdue",IF(H245-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N245" s="51" t="n"/>
@@ -11612,7 +11647,7 @@
         <v/>
       </c>
       <c r="M246" s="58">
-        <f>IF(B246="","",IF(E246="Done","✓ Done",IF(E246="Blocked","Blocked",IF(H246="","No due date",IF(H246&lt;NOW(),"Overdue",IF(H246-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B246="","",IF(E246="Done","Complete",IF(E246="Blocked","Blocked",IF(H246="","No due date",IF(H246&lt;NOW(),"Overdue",IF(H246-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N246" s="51" t="n"/>
@@ -11642,7 +11677,7 @@
         <v/>
       </c>
       <c r="M247" s="58">
-        <f>IF(B247="","",IF(E247="Done","✓ Done",IF(E247="Blocked","Blocked",IF(H247="","No due date",IF(H247&lt;NOW(),"Overdue",IF(H247-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B247="","",IF(E247="Done","Complete",IF(E247="Blocked","Blocked",IF(H247="","No due date",IF(H247&lt;NOW(),"Overdue",IF(H247-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N247" s="51" t="n"/>
@@ -11672,7 +11707,7 @@
         <v/>
       </c>
       <c r="M248" s="58">
-        <f>IF(B248="","",IF(E248="Done","✓ Done",IF(E248="Blocked","Blocked",IF(H248="","No due date",IF(H248&lt;NOW(),"Overdue",IF(H248-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B248="","",IF(E248="Done","Complete",IF(E248="Blocked","Blocked",IF(H248="","No due date",IF(H248&lt;NOW(),"Overdue",IF(H248-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N248" s="51" t="n"/>
@@ -11702,7 +11737,7 @@
         <v/>
       </c>
       <c r="M249" s="58">
-        <f>IF(B249="","",IF(E249="Done","✓ Done",IF(E249="Blocked","Blocked",IF(H249="","No due date",IF(H249&lt;NOW(),"Overdue",IF(H249-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B249="","",IF(E249="Done","Complete",IF(E249="Blocked","Blocked",IF(H249="","No due date",IF(H249&lt;NOW(),"Overdue",IF(H249-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N249" s="51" t="n"/>
@@ -11732,7 +11767,7 @@
         <v/>
       </c>
       <c r="M250" s="58">
-        <f>IF(B250="","",IF(E250="Done","✓ Done",IF(E250="Blocked","Blocked",IF(H250="","No due date",IF(H250&lt;NOW(),"Overdue",IF(H250-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B250="","",IF(E250="Done","Complete",IF(E250="Blocked","Blocked",IF(H250="","No due date",IF(H250&lt;NOW(),"Overdue",IF(H250-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N250" s="51" t="n"/>
@@ -11762,7 +11797,7 @@
         <v/>
       </c>
       <c r="M251" s="58">
-        <f>IF(B251="","",IF(E251="Done","✓ Done",IF(E251="Blocked","Blocked",IF(H251="","No due date",IF(H251&lt;NOW(),"Overdue",IF(H251-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B251="","",IF(E251="Done","Complete",IF(E251="Blocked","Blocked",IF(H251="","No due date",IF(H251&lt;NOW(),"Overdue",IF(H251-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N251" s="51" t="n"/>
@@ -11792,7 +11827,7 @@
         <v/>
       </c>
       <c r="M252" s="58">
-        <f>IF(B252="","",IF(E252="Done","✓ Done",IF(E252="Blocked","Blocked",IF(H252="","No due date",IF(H252&lt;NOW(),"Overdue",IF(H252-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B252="","",IF(E252="Done","Complete",IF(E252="Blocked","Blocked",IF(H252="","No due date",IF(H252&lt;NOW(),"Overdue",IF(H252-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N252" s="51" t="n"/>
@@ -11822,7 +11857,7 @@
         <v/>
       </c>
       <c r="M253" s="58">
-        <f>IF(B253="","",IF(E253="Done","✓ Done",IF(E253="Blocked","Blocked",IF(H253="","No due date",IF(H253&lt;NOW(),"Overdue",IF(H253-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B253="","",IF(E253="Done","Complete",IF(E253="Blocked","Blocked",IF(H253="","No due date",IF(H253&lt;NOW(),"Overdue",IF(H253-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N253" s="51" t="n"/>
@@ -11852,7 +11887,7 @@
         <v/>
       </c>
       <c r="M254" s="58">
-        <f>IF(B254="","",IF(E254="Done","✓ Done",IF(E254="Blocked","Blocked",IF(H254="","No due date",IF(H254&lt;NOW(),"Overdue",IF(H254-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B254="","",IF(E254="Done","Complete",IF(E254="Blocked","Blocked",IF(H254="","No due date",IF(H254&lt;NOW(),"Overdue",IF(H254-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N254" s="51" t="n"/>
@@ -11882,7 +11917,7 @@
         <v/>
       </c>
       <c r="M255" s="58">
-        <f>IF(B255="","",IF(E255="Done","✓ Done",IF(E255="Blocked","Blocked",IF(H255="","No due date",IF(H255&lt;NOW(),"Overdue",IF(H255-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B255="","",IF(E255="Done","Complete",IF(E255="Blocked","Blocked",IF(H255="","No due date",IF(H255&lt;NOW(),"Overdue",IF(H255-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N255" s="51" t="n"/>
@@ -11912,7 +11947,7 @@
         <v/>
       </c>
       <c r="M256" s="58">
-        <f>IF(B256="","",IF(E256="Done","✓ Done",IF(E256="Blocked","Blocked",IF(H256="","No due date",IF(H256&lt;NOW(),"Overdue",IF(H256-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B256="","",IF(E256="Done","Complete",IF(E256="Blocked","Blocked",IF(H256="","No due date",IF(H256&lt;NOW(),"Overdue",IF(H256-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N256" s="51" t="n"/>
@@ -11942,7 +11977,7 @@
         <v/>
       </c>
       <c r="M257" s="58">
-        <f>IF(B257="","",IF(E257="Done","✓ Done",IF(E257="Blocked","Blocked",IF(H257="","No due date",IF(H257&lt;NOW(),"Overdue",IF(H257-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B257="","",IF(E257="Done","Complete",IF(E257="Blocked","Blocked",IF(H257="","No due date",IF(H257&lt;NOW(),"Overdue",IF(H257-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N257" s="51" t="n"/>
@@ -11972,7 +12007,7 @@
         <v/>
       </c>
       <c r="M258" s="58">
-        <f>IF(B258="","",IF(E258="Done","✓ Done",IF(E258="Blocked","Blocked",IF(H258="","No due date",IF(H258&lt;NOW(),"Overdue",IF(H258-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B258="","",IF(E258="Done","Complete",IF(E258="Blocked","Blocked",IF(H258="","No due date",IF(H258&lt;NOW(),"Overdue",IF(H258-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N258" s="51" t="n"/>
@@ -12002,7 +12037,7 @@
         <v/>
       </c>
       <c r="M259" s="58">
-        <f>IF(B259="","",IF(E259="Done","✓ Done",IF(E259="Blocked","Blocked",IF(H259="","No due date",IF(H259&lt;NOW(),"Overdue",IF(H259-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B259="","",IF(E259="Done","Complete",IF(E259="Blocked","Blocked",IF(H259="","No due date",IF(H259&lt;NOW(),"Overdue",IF(H259-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N259" s="51" t="n"/>
@@ -12032,7 +12067,7 @@
         <v/>
       </c>
       <c r="M260" s="58">
-        <f>IF(B260="","",IF(E260="Done","✓ Done",IF(E260="Blocked","Blocked",IF(H260="","No due date",IF(H260&lt;NOW(),"Overdue",IF(H260-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B260="","",IF(E260="Done","Complete",IF(E260="Blocked","Blocked",IF(H260="","No due date",IF(H260&lt;NOW(),"Overdue",IF(H260-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N260" s="51" t="n"/>
@@ -12062,7 +12097,7 @@
         <v/>
       </c>
       <c r="M261" s="58">
-        <f>IF(B261="","",IF(E261="Done","✓ Done",IF(E261="Blocked","Blocked",IF(H261="","No due date",IF(H261&lt;NOW(),"Overdue",IF(H261-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B261="","",IF(E261="Done","Complete",IF(E261="Blocked","Blocked",IF(H261="","No due date",IF(H261&lt;NOW(),"Overdue",IF(H261-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N261" s="51" t="n"/>
@@ -12092,7 +12127,7 @@
         <v/>
       </c>
       <c r="M262" s="58">
-        <f>IF(B262="","",IF(E262="Done","✓ Done",IF(E262="Blocked","Blocked",IF(H262="","No due date",IF(H262&lt;NOW(),"Overdue",IF(H262-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B262="","",IF(E262="Done","Complete",IF(E262="Blocked","Blocked",IF(H262="","No due date",IF(H262&lt;NOW(),"Overdue",IF(H262-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N262" s="51" t="n"/>
@@ -12122,7 +12157,7 @@
         <v/>
       </c>
       <c r="M263" s="58">
-        <f>IF(B263="","",IF(E263="Done","✓ Done",IF(E263="Blocked","Blocked",IF(H263="","No due date",IF(H263&lt;NOW(),"Overdue",IF(H263-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B263="","",IF(E263="Done","Complete",IF(E263="Blocked","Blocked",IF(H263="","No due date",IF(H263&lt;NOW(),"Overdue",IF(H263-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N263" s="51" t="n"/>
@@ -12152,7 +12187,7 @@
         <v/>
       </c>
       <c r="M264" s="58">
-        <f>IF(B264="","",IF(E264="Done","✓ Done",IF(E264="Blocked","Blocked",IF(H264="","No due date",IF(H264&lt;NOW(),"Overdue",IF(H264-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B264="","",IF(E264="Done","Complete",IF(E264="Blocked","Blocked",IF(H264="","No due date",IF(H264&lt;NOW(),"Overdue",IF(H264-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N264" s="51" t="n"/>
@@ -12182,7 +12217,7 @@
         <v/>
       </c>
       <c r="M265" s="58">
-        <f>IF(B265="","",IF(E265="Done","✓ Done",IF(E265="Blocked","Blocked",IF(H265="","No due date",IF(H265&lt;NOW(),"Overdue",IF(H265-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B265="","",IF(E265="Done","Complete",IF(E265="Blocked","Blocked",IF(H265="","No due date",IF(H265&lt;NOW(),"Overdue",IF(H265-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N265" s="51" t="n"/>
@@ -12212,7 +12247,7 @@
         <v/>
       </c>
       <c r="M266" s="58">
-        <f>IF(B266="","",IF(E266="Done","✓ Done",IF(E266="Blocked","Blocked",IF(H266="","No due date",IF(H266&lt;NOW(),"Overdue",IF(H266-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B266="","",IF(E266="Done","Complete",IF(E266="Blocked","Blocked",IF(H266="","No due date",IF(H266&lt;NOW(),"Overdue",IF(H266-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N266" s="51" t="n"/>
@@ -12242,7 +12277,7 @@
         <v/>
       </c>
       <c r="M267" s="58">
-        <f>IF(B267="","",IF(E267="Done","✓ Done",IF(E267="Blocked","Blocked",IF(H267="","No due date",IF(H267&lt;NOW(),"Overdue",IF(H267-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B267="","",IF(E267="Done","Complete",IF(E267="Blocked","Blocked",IF(H267="","No due date",IF(H267&lt;NOW(),"Overdue",IF(H267-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N267" s="51" t="n"/>
@@ -12272,7 +12307,7 @@
         <v/>
       </c>
       <c r="M268" s="58">
-        <f>IF(B268="","",IF(E268="Done","✓ Done",IF(E268="Blocked","Blocked",IF(H268="","No due date",IF(H268&lt;NOW(),"Overdue",IF(H268-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B268="","",IF(E268="Done","Complete",IF(E268="Blocked","Blocked",IF(H268="","No due date",IF(H268&lt;NOW(),"Overdue",IF(H268-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N268" s="51" t="n"/>
@@ -12302,7 +12337,7 @@
         <v/>
       </c>
       <c r="M269" s="58">
-        <f>IF(B269="","",IF(E269="Done","✓ Done",IF(E269="Blocked","Blocked",IF(H269="","No due date",IF(H269&lt;NOW(),"Overdue",IF(H269-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B269="","",IF(E269="Done","Complete",IF(E269="Blocked","Blocked",IF(H269="","No due date",IF(H269&lt;NOW(),"Overdue",IF(H269-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N269" s="51" t="n"/>
@@ -12332,7 +12367,7 @@
         <v/>
       </c>
       <c r="M270" s="58">
-        <f>IF(B270="","",IF(E270="Done","✓ Done",IF(E270="Blocked","Blocked",IF(H270="","No due date",IF(H270&lt;NOW(),"Overdue",IF(H270-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B270="","",IF(E270="Done","Complete",IF(E270="Blocked","Blocked",IF(H270="","No due date",IF(H270&lt;NOW(),"Overdue",IF(H270-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N270" s="51" t="n"/>
@@ -12362,7 +12397,7 @@
         <v/>
       </c>
       <c r="M271" s="58">
-        <f>IF(B271="","",IF(E271="Done","✓ Done",IF(E271="Blocked","Blocked",IF(H271="","No due date",IF(H271&lt;NOW(),"Overdue",IF(H271-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B271="","",IF(E271="Done","Complete",IF(E271="Blocked","Blocked",IF(H271="","No due date",IF(H271&lt;NOW(),"Overdue",IF(H271-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N271" s="51" t="n"/>
@@ -12392,7 +12427,7 @@
         <v/>
       </c>
       <c r="M272" s="58">
-        <f>IF(B272="","",IF(E272="Done","✓ Done",IF(E272="Blocked","Blocked",IF(H272="","No due date",IF(H272&lt;NOW(),"Overdue",IF(H272-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B272="","",IF(E272="Done","Complete",IF(E272="Blocked","Blocked",IF(H272="","No due date",IF(H272&lt;NOW(),"Overdue",IF(H272-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N272" s="51" t="n"/>
@@ -12422,7 +12457,7 @@
         <v/>
       </c>
       <c r="M273" s="58">
-        <f>IF(B273="","",IF(E273="Done","✓ Done",IF(E273="Blocked","Blocked",IF(H273="","No due date",IF(H273&lt;NOW(),"Overdue",IF(H273-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B273="","",IF(E273="Done","Complete",IF(E273="Blocked","Blocked",IF(H273="","No due date",IF(H273&lt;NOW(),"Overdue",IF(H273-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N273" s="51" t="n"/>
@@ -12452,7 +12487,7 @@
         <v/>
       </c>
       <c r="M274" s="58">
-        <f>IF(B274="","",IF(E274="Done","✓ Done",IF(E274="Blocked","Blocked",IF(H274="","No due date",IF(H274&lt;NOW(),"Overdue",IF(H274-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B274="","",IF(E274="Done","Complete",IF(E274="Blocked","Blocked",IF(H274="","No due date",IF(H274&lt;NOW(),"Overdue",IF(H274-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N274" s="51" t="n"/>
@@ -12482,7 +12517,7 @@
         <v/>
       </c>
       <c r="M275" s="58">
-        <f>IF(B275="","",IF(E275="Done","✓ Done",IF(E275="Blocked","Blocked",IF(H275="","No due date",IF(H275&lt;NOW(),"Overdue",IF(H275-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B275="","",IF(E275="Done","Complete",IF(E275="Blocked","Blocked",IF(H275="","No due date",IF(H275&lt;NOW(),"Overdue",IF(H275-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N275" s="51" t="n"/>
@@ -12512,7 +12547,7 @@
         <v/>
       </c>
       <c r="M276" s="58">
-        <f>IF(B276="","",IF(E276="Done","✓ Done",IF(E276="Blocked","Blocked",IF(H276="","No due date",IF(H276&lt;NOW(),"Overdue",IF(H276-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B276="","",IF(E276="Done","Complete",IF(E276="Blocked","Blocked",IF(H276="","No due date",IF(H276&lt;NOW(),"Overdue",IF(H276-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N276" s="51" t="n"/>
@@ -12542,7 +12577,7 @@
         <v/>
       </c>
       <c r="M277" s="58">
-        <f>IF(B277="","",IF(E277="Done","✓ Done",IF(E277="Blocked","Blocked",IF(H277="","No due date",IF(H277&lt;NOW(),"Overdue",IF(H277-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B277="","",IF(E277="Done","Complete",IF(E277="Blocked","Blocked",IF(H277="","No due date",IF(H277&lt;NOW(),"Overdue",IF(H277-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N277" s="51" t="n"/>
@@ -12572,7 +12607,7 @@
         <v/>
       </c>
       <c r="M278" s="58">
-        <f>IF(B278="","",IF(E278="Done","✓ Done",IF(E278="Blocked","Blocked",IF(H278="","No due date",IF(H278&lt;NOW(),"Overdue",IF(H278-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B278="","",IF(E278="Done","Complete",IF(E278="Blocked","Blocked",IF(H278="","No due date",IF(H278&lt;NOW(),"Overdue",IF(H278-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N278" s="51" t="n"/>
@@ -12602,7 +12637,7 @@
         <v/>
       </c>
       <c r="M279" s="58">
-        <f>IF(B279="","",IF(E279="Done","✓ Done",IF(E279="Blocked","Blocked",IF(H279="","No due date",IF(H279&lt;NOW(),"Overdue",IF(H279-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B279="","",IF(E279="Done","Complete",IF(E279="Blocked","Blocked",IF(H279="","No due date",IF(H279&lt;NOW(),"Overdue",IF(H279-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N279" s="51" t="n"/>
@@ -12632,7 +12667,7 @@
         <v/>
       </c>
       <c r="M280" s="58">
-        <f>IF(B280="","",IF(E280="Done","✓ Done",IF(E280="Blocked","Blocked",IF(H280="","No due date",IF(H280&lt;NOW(),"Overdue",IF(H280-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B280="","",IF(E280="Done","Complete",IF(E280="Blocked","Blocked",IF(H280="","No due date",IF(H280&lt;NOW(),"Overdue",IF(H280-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N280" s="51" t="n"/>
@@ -12662,7 +12697,7 @@
         <v/>
       </c>
       <c r="M281" s="58">
-        <f>IF(B281="","",IF(E281="Done","✓ Done",IF(E281="Blocked","Blocked",IF(H281="","No due date",IF(H281&lt;NOW(),"Overdue",IF(H281-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B281="","",IF(E281="Done","Complete",IF(E281="Blocked","Blocked",IF(H281="","No due date",IF(H281&lt;NOW(),"Overdue",IF(H281-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N281" s="51" t="n"/>
@@ -12692,7 +12727,7 @@
         <v/>
       </c>
       <c r="M282" s="58">
-        <f>IF(B282="","",IF(E282="Done","✓ Done",IF(E282="Blocked","Blocked",IF(H282="","No due date",IF(H282&lt;NOW(),"Overdue",IF(H282-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B282="","",IF(E282="Done","Complete",IF(E282="Blocked","Blocked",IF(H282="","No due date",IF(H282&lt;NOW(),"Overdue",IF(H282-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N282" s="51" t="n"/>
@@ -12722,7 +12757,7 @@
         <v/>
       </c>
       <c r="M283" s="58">
-        <f>IF(B283="","",IF(E283="Done","✓ Done",IF(E283="Blocked","Blocked",IF(H283="","No due date",IF(H283&lt;NOW(),"Overdue",IF(H283-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B283="","",IF(E283="Done","Complete",IF(E283="Blocked","Blocked",IF(H283="","No due date",IF(H283&lt;NOW(),"Overdue",IF(H283-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N283" s="51" t="n"/>
@@ -12752,7 +12787,7 @@
         <v/>
       </c>
       <c r="M284" s="58">
-        <f>IF(B284="","",IF(E284="Done","✓ Done",IF(E284="Blocked","Blocked",IF(H284="","No due date",IF(H284&lt;NOW(),"Overdue",IF(H284-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B284="","",IF(E284="Done","Complete",IF(E284="Blocked","Blocked",IF(H284="","No due date",IF(H284&lt;NOW(),"Overdue",IF(H284-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N284" s="51" t="n"/>
@@ -12782,7 +12817,7 @@
         <v/>
       </c>
       <c r="M285" s="58">
-        <f>IF(B285="","",IF(E285="Done","✓ Done",IF(E285="Blocked","Blocked",IF(H285="","No due date",IF(H285&lt;NOW(),"Overdue",IF(H285-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B285="","",IF(E285="Done","Complete",IF(E285="Blocked","Blocked",IF(H285="","No due date",IF(H285&lt;NOW(),"Overdue",IF(H285-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N285" s="51" t="n"/>
@@ -12812,7 +12847,7 @@
         <v/>
       </c>
       <c r="M286" s="58">
-        <f>IF(B286="","",IF(E286="Done","✓ Done",IF(E286="Blocked","Blocked",IF(H286="","No due date",IF(H286&lt;NOW(),"Overdue",IF(H286-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B286="","",IF(E286="Done","Complete",IF(E286="Blocked","Blocked",IF(H286="","No due date",IF(H286&lt;NOW(),"Overdue",IF(H286-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N286" s="51" t="n"/>
@@ -12842,7 +12877,7 @@
         <v/>
       </c>
       <c r="M287" s="58">
-        <f>IF(B287="","",IF(E287="Done","✓ Done",IF(E287="Blocked","Blocked",IF(H287="","No due date",IF(H287&lt;NOW(),"Overdue",IF(H287-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B287="","",IF(E287="Done","Complete",IF(E287="Blocked","Blocked",IF(H287="","No due date",IF(H287&lt;NOW(),"Overdue",IF(H287-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N287" s="51" t="n"/>
@@ -12872,7 +12907,7 @@
         <v/>
       </c>
       <c r="M288" s="58">
-        <f>IF(B288="","",IF(E288="Done","✓ Done",IF(E288="Blocked","Blocked",IF(H288="","No due date",IF(H288&lt;NOW(),"Overdue",IF(H288-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B288="","",IF(E288="Done","Complete",IF(E288="Blocked","Blocked",IF(H288="","No due date",IF(H288&lt;NOW(),"Overdue",IF(H288-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N288" s="51" t="n"/>
@@ -12902,7 +12937,7 @@
         <v/>
       </c>
       <c r="M289" s="58">
-        <f>IF(B289="","",IF(E289="Done","✓ Done",IF(E289="Blocked","Blocked",IF(H289="","No due date",IF(H289&lt;NOW(),"Overdue",IF(H289-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B289="","",IF(E289="Done","Complete",IF(E289="Blocked","Blocked",IF(H289="","No due date",IF(H289&lt;NOW(),"Overdue",IF(H289-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N289" s="51" t="n"/>
@@ -12932,7 +12967,7 @@
         <v/>
       </c>
       <c r="M290" s="58">
-        <f>IF(B290="","",IF(E290="Done","✓ Done",IF(E290="Blocked","Blocked",IF(H290="","No due date",IF(H290&lt;NOW(),"Overdue",IF(H290-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B290="","",IF(E290="Done","Complete",IF(E290="Blocked","Blocked",IF(H290="","No due date",IF(H290&lt;NOW(),"Overdue",IF(H290-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N290" s="51" t="n"/>
@@ -12962,7 +12997,7 @@
         <v/>
       </c>
       <c r="M291" s="58">
-        <f>IF(B291="","",IF(E291="Done","✓ Done",IF(E291="Blocked","Blocked",IF(H291="","No due date",IF(H291&lt;NOW(),"Overdue",IF(H291-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B291="","",IF(E291="Done","Complete",IF(E291="Blocked","Blocked",IF(H291="","No due date",IF(H291&lt;NOW(),"Overdue",IF(H291-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N291" s="51" t="n"/>
@@ -12992,7 +13027,7 @@
         <v/>
       </c>
       <c r="M292" s="58">
-        <f>IF(B292="","",IF(E292="Done","✓ Done",IF(E292="Blocked","Blocked",IF(H292="","No due date",IF(H292&lt;NOW(),"Overdue",IF(H292-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B292="","",IF(E292="Done","Complete",IF(E292="Blocked","Blocked",IF(H292="","No due date",IF(H292&lt;NOW(),"Overdue",IF(H292-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N292" s="51" t="n"/>
@@ -13022,7 +13057,7 @@
         <v/>
       </c>
       <c r="M293" s="58">
-        <f>IF(B293="","",IF(E293="Done","✓ Done",IF(E293="Blocked","Blocked",IF(H293="","No due date",IF(H293&lt;NOW(),"Overdue",IF(H293-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B293="","",IF(E293="Done","Complete",IF(E293="Blocked","Blocked",IF(H293="","No due date",IF(H293&lt;NOW(),"Overdue",IF(H293-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N293" s="51" t="n"/>
@@ -13052,7 +13087,7 @@
         <v/>
       </c>
       <c r="M294" s="58">
-        <f>IF(B294="","",IF(E294="Done","✓ Done",IF(E294="Blocked","Blocked",IF(H294="","No due date",IF(H294&lt;NOW(),"Overdue",IF(H294-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B294="","",IF(E294="Done","Complete",IF(E294="Blocked","Blocked",IF(H294="","No due date",IF(H294&lt;NOW(),"Overdue",IF(H294-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N294" s="51" t="n"/>
@@ -13082,7 +13117,7 @@
         <v/>
       </c>
       <c r="M295" s="58">
-        <f>IF(B295="","",IF(E295="Done","✓ Done",IF(E295="Blocked","Blocked",IF(H295="","No due date",IF(H295&lt;NOW(),"Overdue",IF(H295-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B295="","",IF(E295="Done","Complete",IF(E295="Blocked","Blocked",IF(H295="","No due date",IF(H295&lt;NOW(),"Overdue",IF(H295-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N295" s="51" t="n"/>
@@ -13112,7 +13147,7 @@
         <v/>
       </c>
       <c r="M296" s="58">
-        <f>IF(B296="","",IF(E296="Done","✓ Done",IF(E296="Blocked","Blocked",IF(H296="","No due date",IF(H296&lt;NOW(),"Overdue",IF(H296-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B296="","",IF(E296="Done","Complete",IF(E296="Blocked","Blocked",IF(H296="","No due date",IF(H296&lt;NOW(),"Overdue",IF(H296-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N296" s="51" t="n"/>
@@ -13142,7 +13177,7 @@
         <v/>
       </c>
       <c r="M297" s="58">
-        <f>IF(B297="","",IF(E297="Done","✓ Done",IF(E297="Blocked","Blocked",IF(H297="","No due date",IF(H297&lt;NOW(),"Overdue",IF(H297-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B297="","",IF(E297="Done","Complete",IF(E297="Blocked","Blocked",IF(H297="","No due date",IF(H297&lt;NOW(),"Overdue",IF(H297-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N297" s="51" t="n"/>
@@ -13172,7 +13207,7 @@
         <v/>
       </c>
       <c r="M298" s="58">
-        <f>IF(B298="","",IF(E298="Done","✓ Done",IF(E298="Blocked","Blocked",IF(H298="","No due date",IF(H298&lt;NOW(),"Overdue",IF(H298-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B298="","",IF(E298="Done","Complete",IF(E298="Blocked","Blocked",IF(H298="","No due date",IF(H298&lt;NOW(),"Overdue",IF(H298-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N298" s="51" t="n"/>
@@ -13202,7 +13237,7 @@
         <v/>
       </c>
       <c r="M299" s="58">
-        <f>IF(B299="","",IF(E299="Done","✓ Done",IF(E299="Blocked","Blocked",IF(H299="","No due date",IF(H299&lt;NOW(),"Overdue",IF(H299-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B299="","",IF(E299="Done","Complete",IF(E299="Blocked","Blocked",IF(H299="","No due date",IF(H299&lt;NOW(),"Overdue",IF(H299-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N299" s="51" t="n"/>
@@ -13232,7 +13267,7 @@
         <v/>
       </c>
       <c r="M300" s="58">
-        <f>IF(B300="","",IF(E300="Done","✓ Done",IF(E300="Blocked","Blocked",IF(H300="","No due date",IF(H300&lt;NOW(),"Overdue",IF(H300-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B300="","",IF(E300="Done","Complete",IF(E300="Blocked","Blocked",IF(H300="","No due date",IF(H300&lt;NOW(),"Overdue",IF(H300-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N300" s="51" t="n"/>
@@ -13262,7 +13297,7 @@
         <v/>
       </c>
       <c r="M301" s="58">
-        <f>IF(B301="","",IF(E301="Done","✓ Done",IF(E301="Blocked","Blocked",IF(H301="","No due date",IF(H301&lt;NOW(),"Overdue",IF(H301-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B301="","",IF(E301="Done","Complete",IF(E301="Blocked","Blocked",IF(H301="","No due date",IF(H301&lt;NOW(),"Overdue",IF(H301-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N301" s="51" t="n"/>
@@ -13292,7 +13327,7 @@
         <v/>
       </c>
       <c r="M302" s="58">
-        <f>IF(B302="","",IF(E302="Done","✓ Done",IF(E302="Blocked","Blocked",IF(H302="","No due date",IF(H302&lt;NOW(),"Overdue",IF(H302-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B302="","",IF(E302="Done","Complete",IF(E302="Blocked","Blocked",IF(H302="","No due date",IF(H302&lt;NOW(),"Overdue",IF(H302-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N302" s="51" t="n"/>
@@ -13322,7 +13357,7 @@
         <v/>
       </c>
       <c r="M303" s="58">
-        <f>IF(B303="","",IF(E303="Done","✓ Done",IF(E303="Blocked","Blocked",IF(H303="","No due date",IF(H303&lt;NOW(),"Overdue",IF(H303-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B303="","",IF(E303="Done","Complete",IF(E303="Blocked","Blocked",IF(H303="","No due date",IF(H303&lt;NOW(),"Overdue",IF(H303-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N303" s="51" t="n"/>
@@ -13352,7 +13387,7 @@
         <v/>
       </c>
       <c r="M304" s="58">
-        <f>IF(B304="","",IF(E304="Done","✓ Done",IF(E304="Blocked","Blocked",IF(H304="","No due date",IF(H304&lt;NOW(),"Overdue",IF(H304-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B304="","",IF(E304="Done","Complete",IF(E304="Blocked","Blocked",IF(H304="","No due date",IF(H304&lt;NOW(),"Overdue",IF(H304-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N304" s="51" t="n"/>
@@ -13382,7 +13417,7 @@
         <v/>
       </c>
       <c r="M305" s="58">
-        <f>IF(B305="","",IF(E305="Done","✓ Done",IF(E305="Blocked","Blocked",IF(H305="","No due date",IF(H305&lt;NOW(),"Overdue",IF(H305-NOW()&lt;=3,"Due soon","On track"))))))</f>
+        <f>IF(B305="","",IF(E305="Done","Complete",IF(E305="Blocked","Blocked",IF(H305="","No due date",IF(H305&lt;NOW(),"Overdue",IF(H305-NOW()&lt;=3,"Due soon","On track"))))))</f>
         <v/>
       </c>
       <c r="N305" s="51" t="n"/>
@@ -13395,19 +13430,19 @@
   </sheetData>
   <autoFilter ref="A5:O305"/>
   <conditionalFormatting sqref="E6:E305">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="6">
       <formula>"Not started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="7">
       <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="8">
       <formula>"In review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="9">
       <formula>"Blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="10">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13421,29 +13456,29 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M6:M305">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="9">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="12">
       <formula>"Overdue"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="10">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="13">
       <formula>"Due soon"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="9">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="12">
       <formula>"Blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="14">
       <formula>"On track"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="12">
-      <formula>"✓ Done"</formula>
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="15">
+      <formula>"Complete"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F6:F305">
-    <cfRule type="cellIs" priority="12" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="4">
       <formula>"Critical"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:B305">
-    <cfRule type="expression" priority="13" dxfId="13">
+    <cfRule type="expression" priority="13" dxfId="16">
       <formula>$E6="Done"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13589,7 +13624,7 @@
         <v/>
       </c>
       <c r="H6" s="58">
-        <f>IF(B6="","",IF(AND(E6&gt;0,F6=E6),"✓ Complete",IF(C6="","Planned",IF(C6&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B6="","",IF(AND(E6&gt;0,F6=E6),"Complete",IF(C6="","Planned",IF(C6&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I6" s="59" t="inlineStr">
@@ -13623,7 +13658,7 @@
         <v/>
       </c>
       <c r="H7" s="58">
-        <f>IF(B7="","",IF(AND(E7&gt;0,F7=E7),"✓ Complete",IF(C7="","Planned",IF(C7&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B7="","",IF(AND(E7&gt;0,F7=E7),"Complete",IF(C7="","Planned",IF(C7&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I7" s="59" t="inlineStr">
@@ -13657,7 +13692,7 @@
         <v/>
       </c>
       <c r="H8" s="58">
-        <f>IF(B8="","",IF(AND(E8&gt;0,F8=E8),"✓ Complete",IF(C8="","Planned",IF(C8&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B8="","",IF(AND(E8&gt;0,F8=E8),"Complete",IF(C8="","Planned",IF(C8&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I8" s="59" t="inlineStr"/>
@@ -13687,7 +13722,7 @@
         <v/>
       </c>
       <c r="H9" s="58">
-        <f>IF(B9="","",IF(AND(E9&gt;0,F9=E9),"✓ Complete",IF(C9="","Planned",IF(C9&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B9="","",IF(AND(E9&gt;0,F9=E9),"Complete",IF(C9="","Planned",IF(C9&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I9" s="59" t="inlineStr"/>
@@ -13717,7 +13752,7 @@
         <v/>
       </c>
       <c r="H10" s="58">
-        <f>IF(B10="","",IF(AND(E10&gt;0,F10=E10),"✓ Complete",IF(C10="","Planned",IF(C10&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B10="","",IF(AND(E10&gt;0,F10=E10),"Complete",IF(C10="","Planned",IF(C10&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I10" s="59" t="inlineStr">
@@ -13747,7 +13782,7 @@
         <v/>
       </c>
       <c r="H11" s="58">
-        <f>IF(B11="","",IF(AND(E11&gt;0,F11=E11),"✓ Complete",IF(C11="","Planned",IF(C11&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B11="","",IF(AND(E11&gt;0,F11=E11),"Complete",IF(C11="","Planned",IF(C11&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I11" s="59" t="n"/>
@@ -13773,7 +13808,7 @@
         <v/>
       </c>
       <c r="H12" s="58">
-        <f>IF(B12="","",IF(AND(E12&gt;0,F12=E12),"✓ Complete",IF(C12="","Planned",IF(C12&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B12="","",IF(AND(E12&gt;0,F12=E12),"Complete",IF(C12="","Planned",IF(C12&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I12" s="59" t="n"/>
@@ -13799,7 +13834,7 @@
         <v/>
       </c>
       <c r="H13" s="58">
-        <f>IF(B13="","",IF(AND(E13&gt;0,F13=E13),"✓ Complete",IF(C13="","Planned",IF(C13&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B13="","",IF(AND(E13&gt;0,F13=E13),"Complete",IF(C13="","Planned",IF(C13&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I13" s="59" t="n"/>
@@ -13825,7 +13860,7 @@
         <v/>
       </c>
       <c r="H14" s="58">
-        <f>IF(B14="","",IF(AND(E14&gt;0,F14=E14),"✓ Complete",IF(C14="","Planned",IF(C14&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B14="","",IF(AND(E14&gt;0,F14=E14),"Complete",IF(C14="","Planned",IF(C14&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I14" s="59" t="n"/>
@@ -13851,7 +13886,7 @@
         <v/>
       </c>
       <c r="H15" s="58">
-        <f>IF(B15="","",IF(AND(E15&gt;0,F15=E15),"✓ Complete",IF(C15="","Planned",IF(C15&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B15="","",IF(AND(E15&gt;0,F15=E15),"Complete",IF(C15="","Planned",IF(C15&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I15" s="59" t="n"/>
@@ -13877,7 +13912,7 @@
         <v/>
       </c>
       <c r="H16" s="58">
-        <f>IF(B16="","",IF(AND(E16&gt;0,F16=E16),"✓ Complete",IF(C16="","Planned",IF(C16&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B16="","",IF(AND(E16&gt;0,F16=E16),"Complete",IF(C16="","Planned",IF(C16&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I16" s="59" t="n"/>
@@ -13903,7 +13938,7 @@
         <v/>
       </c>
       <c r="H17" s="58">
-        <f>IF(B17="","",IF(AND(E17&gt;0,F17=E17),"✓ Complete",IF(C17="","Planned",IF(C17&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B17="","",IF(AND(E17&gt;0,F17=E17),"Complete",IF(C17="","Planned",IF(C17&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I17" s="59" t="n"/>
@@ -13929,7 +13964,7 @@
         <v/>
       </c>
       <c r="H18" s="58">
-        <f>IF(B18="","",IF(AND(E18&gt;0,F18=E18),"✓ Complete",IF(C18="","Planned",IF(C18&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B18="","",IF(AND(E18&gt;0,F18=E18),"Complete",IF(C18="","Planned",IF(C18&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I18" s="59" t="n"/>
@@ -13955,7 +13990,7 @@
         <v/>
       </c>
       <c r="H19" s="58">
-        <f>IF(B19="","",IF(AND(E19&gt;0,F19=E19),"✓ Complete",IF(C19="","Planned",IF(C19&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B19="","",IF(AND(E19&gt;0,F19=E19),"Complete",IF(C19="","Planned",IF(C19&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I19" s="59" t="n"/>
@@ -13981,7 +14016,7 @@
         <v/>
       </c>
       <c r="H20" s="58">
-        <f>IF(B20="","",IF(AND(E20&gt;0,F20=E20),"✓ Complete",IF(C20="","Planned",IF(C20&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B20="","",IF(AND(E20&gt;0,F20=E20),"Complete",IF(C20="","Planned",IF(C20&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I20" s="59" t="n"/>
@@ -14007,7 +14042,7 @@
         <v/>
       </c>
       <c r="H21" s="58">
-        <f>IF(B21="","",IF(AND(E21&gt;0,F21=E21),"✓ Complete",IF(C21="","Planned",IF(C21&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B21="","",IF(AND(E21&gt;0,F21=E21),"Complete",IF(C21="","Planned",IF(C21&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I21" s="59" t="n"/>
@@ -14033,7 +14068,7 @@
         <v/>
       </c>
       <c r="H22" s="58">
-        <f>IF(B22="","",IF(AND(E22&gt;0,F22=E22),"✓ Complete",IF(C22="","Planned",IF(C22&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B22="","",IF(AND(E22&gt;0,F22=E22),"Complete",IF(C22="","Planned",IF(C22&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I22" s="59" t="n"/>
@@ -14059,7 +14094,7 @@
         <v/>
       </c>
       <c r="H23" s="58">
-        <f>IF(B23="","",IF(AND(E23&gt;0,F23=E23),"✓ Complete",IF(C23="","Planned",IF(C23&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B23="","",IF(AND(E23&gt;0,F23=E23),"Complete",IF(C23="","Planned",IF(C23&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I23" s="59" t="n"/>
@@ -14085,7 +14120,7 @@
         <v/>
       </c>
       <c r="H24" s="58">
-        <f>IF(B24="","",IF(AND(E24&gt;0,F24=E24),"✓ Complete",IF(C24="","Planned",IF(C24&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B24="","",IF(AND(E24&gt;0,F24=E24),"Complete",IF(C24="","Planned",IF(C24&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I24" s="59" t="n"/>
@@ -14111,7 +14146,7 @@
         <v/>
       </c>
       <c r="H25" s="58">
-        <f>IF(B25="","",IF(AND(E25&gt;0,F25=E25),"✓ Complete",IF(C25="","Planned",IF(C25&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B25="","",IF(AND(E25&gt;0,F25=E25),"Complete",IF(C25="","Planned",IF(C25&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I25" s="59" t="n"/>
@@ -14137,7 +14172,7 @@
         <v/>
       </c>
       <c r="H26" s="58">
-        <f>IF(B26="","",IF(AND(E26&gt;0,F26=E26),"✓ Complete",IF(C26="","Planned",IF(C26&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B26="","",IF(AND(E26&gt;0,F26=E26),"Complete",IF(C26="","Planned",IF(C26&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I26" s="59" t="n"/>
@@ -14163,7 +14198,7 @@
         <v/>
       </c>
       <c r="H27" s="58">
-        <f>IF(B27="","",IF(AND(E27&gt;0,F27=E27),"✓ Complete",IF(C27="","Planned",IF(C27&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B27="","",IF(AND(E27&gt;0,F27=E27),"Complete",IF(C27="","Planned",IF(C27&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I27" s="59" t="n"/>
@@ -14189,7 +14224,7 @@
         <v/>
       </c>
       <c r="H28" s="58">
-        <f>IF(B28="","",IF(AND(E28&gt;0,F28=E28),"✓ Complete",IF(C28="","Planned",IF(C28&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B28="","",IF(AND(E28&gt;0,F28=E28),"Complete",IF(C28="","Planned",IF(C28&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I28" s="59" t="n"/>
@@ -14215,7 +14250,7 @@
         <v/>
       </c>
       <c r="H29" s="58">
-        <f>IF(B29="","",IF(AND(E29&gt;0,F29=E29),"✓ Complete",IF(C29="","Planned",IF(C29&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B29="","",IF(AND(E29&gt;0,F29=E29),"Complete",IF(C29="","Planned",IF(C29&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I29" s="59" t="n"/>
@@ -14241,7 +14276,7 @@
         <v/>
       </c>
       <c r="H30" s="58">
-        <f>IF(B30="","",IF(AND(E30&gt;0,F30=E30),"✓ Complete",IF(C30="","Planned",IF(C30&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B30="","",IF(AND(E30&gt;0,F30=E30),"Complete",IF(C30="","Planned",IF(C30&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I30" s="59" t="n"/>
@@ -14267,7 +14302,7 @@
         <v/>
       </c>
       <c r="H31" s="58">
-        <f>IF(B31="","",IF(AND(E31&gt;0,F31=E31),"✓ Complete",IF(C31="","Planned",IF(C31&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B31="","",IF(AND(E31&gt;0,F31=E31),"Complete",IF(C31="","Planned",IF(C31&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I31" s="59" t="n"/>
@@ -14293,7 +14328,7 @@
         <v/>
       </c>
       <c r="H32" s="58">
-        <f>IF(B32="","",IF(AND(E32&gt;0,F32=E32),"✓ Complete",IF(C32="","Planned",IF(C32&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B32="","",IF(AND(E32&gt;0,F32=E32),"Complete",IF(C32="","Planned",IF(C32&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I32" s="59" t="n"/>
@@ -14319,7 +14354,7 @@
         <v/>
       </c>
       <c r="H33" s="58">
-        <f>IF(B33="","",IF(AND(E33&gt;0,F33=E33),"✓ Complete",IF(C33="","Planned",IF(C33&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B33="","",IF(AND(E33&gt;0,F33=E33),"Complete",IF(C33="","Planned",IF(C33&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I33" s="59" t="n"/>
@@ -14345,7 +14380,7 @@
         <v/>
       </c>
       <c r="H34" s="58">
-        <f>IF(B34="","",IF(AND(E34&gt;0,F34=E34),"✓ Complete",IF(C34="","Planned",IF(C34&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B34="","",IF(AND(E34&gt;0,F34=E34),"Complete",IF(C34="","Planned",IF(C34&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I34" s="59" t="n"/>
@@ -14371,7 +14406,7 @@
         <v/>
       </c>
       <c r="H35" s="58">
-        <f>IF(B35="","",IF(AND(E35&gt;0,F35=E35),"✓ Complete",IF(C35="","Planned",IF(C35&lt;NOW(),"Late","On track"))))</f>
+        <f>IF(B35="","",IF(AND(E35&gt;0,F35=E35),"Complete",IF(C35="","Planned",IF(C35&lt;NOW(),"Late","On track"))))</f>
         <v/>
       </c>
       <c r="I35" s="59" t="n"/>
@@ -14387,13 +14422,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6:H35">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="9">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="12">
       <formula>"Late"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="12">
-      <formula>"✓ Complete"</formula>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="15">
+      <formula>"Complete"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="11">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="14">
       <formula>"On track"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23762,39 +23797,39 @@
     <mergeCell ref="G3:K3"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:CK85">
-    <cfRule type="expression" priority="1" dxfId="14" stopIfTrue="1">
+    <cfRule type="expression" priority="1" dxfId="17" stopIfTrue="1">
       <formula>AND(AND($A6&lt;&gt;"",F$5&gt;=INT($D6),F$5&lt;=INT($E6)),$C6="Done")</formula>
     </cfRule>
-    <cfRule type="expression" priority="2" dxfId="15" stopIfTrue="1">
+    <cfRule type="expression" priority="2" dxfId="18" stopIfTrue="1">
       <formula>AND(AND($A6&lt;&gt;"",F$5&gt;=INT($D6),F$5&lt;=INT($E6)),$E6&lt;NOW())</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="16" stopIfTrue="1">
+    <cfRule type="expression" priority="3" dxfId="19" stopIfTrue="1">
       <formula>AND(AND($A6&lt;&gt;"",F$5&gt;=INT($D6),F$5&lt;=INT($E6)),$C6="Blocked")</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="17" stopIfTrue="1">
+    <cfRule type="expression" priority="4" dxfId="20" stopIfTrue="1">
       <formula>AND($A6&lt;&gt;"",F$5&gt;=INT($D6),F$5&lt;=INT($E6))</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="18">
+    <cfRule type="expression" priority="5" dxfId="21">
       <formula>F$5=TODAY()</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="19">
+    <cfRule type="expression" priority="6" dxfId="22">
       <formula>WEEKDAY(F$5,2)&gt;5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6:C85">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="6">
       <formula>"Not started"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="7">
       <formula>"In progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="8">
       <formula>"In review"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="9">
       <formula>"Blocked"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="10">
       <formula>"Done"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -23918,7 +23953,7 @@
       </c>
       <c r="G6" s="77" t="inlineStr">
         <is>
-          <t>🙂 Good</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="H6" s="77" t="inlineStr">
@@ -28920,7 +28955,7 @@
   </sheetData>
   <autoFilter ref="A5:H505"/>
   <conditionalFormatting sqref="E6:E505">
-    <cfRule type="expression" priority="1" dxfId="9">
+    <cfRule type="expression" priority="1" dxfId="12">
       <formula>AND(E6&lt;&gt;"",E6&lt;&gt;"-",E6&lt;&gt;"—",LOWER(E6)&lt;&gt;"none")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -34402,10 +34437,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H9:Q158">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="7">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="10">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="7">
       <formula>"In progress"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -36838,12 +36873,12 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:G105">
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
       <formula>"High"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B6:J105">
-    <cfRule type="expression" priority="3" dxfId="20">
+    <cfRule type="expression" priority="3" dxfId="23">
       <formula>$J6="Closed"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>